<commit_message>
fix(curriculum): complete D3+ verification, remove LaTeX math, enforce ASCII diagrams, resolve 7 duplicate algorithms, and sync Excel/QA
</commit_message>
<xml_diff>
--- a/SWEA_알고리즘_문제집_커리큘럼.xlsx
+++ b/SWEA_알고리즘_문제집_커리큘럼.xlsx
@@ -168,7 +168,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -204,44 +204,11 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="001F497D"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BDD7EE"/>
-      </right>
-      <top style="medium">
-        <color rgb="001F497D"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BDD7EE"/>
-      </right>
-      <top style="medium">
-        <color rgb="001F497D"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="001F497D"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -337,7 +304,6 @@
     <xf numFmtId="0" fontId="6" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -763,31 +729,28 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>총 개발 문항</t>
         </is>
       </c>
-      <c r="B4" s="33" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>기초 D2 (미세사다리)</t>
         </is>
       </c>
-      <c r="D4" s="33" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>실전 D3 (20인스토리)</t>
         </is>
       </c>
-      <c r="F4" s="33" t="n"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>심화 D4 (복합제약)</t>
         </is>
       </c>
-      <c r="H4" s="33" t="n"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>전문가 D5 (B형Pro)</t>
@@ -798,7 +761,6 @@
           <t>규격 통과율</t>
         </is>
       </c>
-      <c r="K4" s="33" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -806,25 +768,21 @@
           <t>358개</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>120개</t>
         </is>
       </c>
-      <c r="D5" s="33" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>114개</t>
         </is>
       </c>
-      <c r="F5" s="33" t="n"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
           <t>116개</t>
         </is>
       </c>
-      <c r="H5" s="33" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>8개</t>
@@ -835,33 +793,29 @@
           <t>100% PASS</t>
         </is>
       </c>
-      <c r="K5" s="33" t="n"/>
-    </row>
+    </row>
+    <row r="6"/>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>🚀 총 대상 문항</t>
         </is>
       </c>
-      <c r="B7" s="33" t="n"/>
       <c r="C7" s="5" t="inlineStr">
         <is>
           <t>✅ 업로드 완료</t>
         </is>
       </c>
-      <c r="D7" s="33" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>⏳ 검토/진행중</t>
         </is>
       </c>
-      <c r="F7" s="33" t="n"/>
       <c r="G7" s="5" t="inlineStr">
         <is>
           <t>⬜ 업로드 대기</t>
         </is>
       </c>
-      <c r="H7" s="33" t="n"/>
       <c r="I7" s="5" t="inlineStr">
         <is>
           <t>SSAFY 연계 클립</t>
@@ -872,7 +826,6 @@
           <t>업로드 달성률</t>
         </is>
       </c>
-      <c r="K7" s="33" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -880,22 +833,18 @@
           <t>358개</t>
         </is>
       </c>
-      <c r="B8" s="33" t="n"/>
       <c r="C8" s="6">
         <f>COUNTIF('📋 전체_문제_목록'!E2:E359, "✅ 업로드 완료")</f>
         <v/>
       </c>
-      <c r="D8" s="33" t="n"/>
       <c r="E8" s="6">
         <f>COUNTIF('📋 전체_문제_목록'!E2:E359, "⏳ 검토중")</f>
         <v/>
       </c>
-      <c r="F8" s="33" t="n"/>
       <c r="G8" s="6">
         <f>COUNTIF('📋 전체_문제_목록'!E2:E359, "⬜ 대기")</f>
         <v/>
       </c>
-      <c r="H8" s="33" t="n"/>
       <c r="I8" s="6" t="inlineStr">
         <is>
           <t>86개 클립</t>
@@ -905,8 +854,8 @@
         <f>COUNTIF('📋 전체_문제_목록'!E2:E359, "✅ 업로드 완료")/358</f>
         <v/>
       </c>
-      <c r="K8" s="33" t="n"/>
-    </row>
+    </row>
+    <row r="9"/>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
@@ -2479,43 +2428,38 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>총 강의 클립</t>
         </is>
       </c>
-      <c r="B4" s="33" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>연계 매칭 문항</t>
         </is>
       </c>
-      <c r="D4" s="33" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>업로드 완료</t>
         </is>
       </c>
-      <c r="F4" s="33" t="n"/>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>검토 및 진행중</t>
         </is>
       </c>
-      <c r="H4" s="33" t="n"/>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>업로드 대기</t>
         </is>
       </c>
-      <c r="J4" s="33" t="n"/>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>로드맵 진척도</t>
         </is>
       </c>
-      <c r="L4" s="33" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -2523,34 +2467,30 @@
           <t>86개</t>
         </is>
       </c>
-      <c r="B5" s="33" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>86문제</t>
         </is>
       </c>
-      <c r="D5" s="33" t="n"/>
       <c r="E5" s="4">
         <f>COUNTIF(I9:I94, "✅ 업로드 완료")</f>
         <v/>
       </c>
-      <c r="F5" s="33" t="n"/>
       <c r="G5" s="4">
         <f>COUNTIF(I9:I94, "⏳ 검토중")</f>
         <v/>
       </c>
-      <c r="H5" s="33" t="n"/>
       <c r="I5" s="4">
         <f>COUNTIF(I9:I94, "⬜ 대기")</f>
         <v/>
       </c>
-      <c r="J5" s="33" t="n"/>
       <c r="K5" s="21">
         <f>COUNTIF(I9:I94, "✅ 업로드 완료")/86</f>
         <v/>
       </c>
-      <c r="L5" s="33" t="n"/>
-    </row>
+    </row>
+    <row r="6"/>
+    <row r="7"/>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -8036,7 +7976,7 @@
       </c>
       <c r="M3" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 격자 미로가 주어진다. 미로에서 1은 이동할 수 있는 칸을 나타내고, 0은 이동할 수 없는 벽을 나타낸다.</t>
+          <t>너비 우선 탐색(BFS) 알고리즘 개념 및 동작 원리 설명: 너비 우선 탐색(BFS)은 시작 위치에서 출발하여 거리가 1인 칸부터 큐(Queue)에 넣어 가까운 곳부터 차례대로 탐색하는 대표적인 최단 경로 탐색 원리...</t>
         </is>
       </c>
       <c r="N3" s="17" t="inlineStr">
@@ -8246,7 +8186,7 @@
       </c>
       <c r="M6" s="12" t="inlineStr">
         <is>
-          <t>수빈이는 동생과 숨바꼭질을 하고 있다. 수빈이는 현재 점 N(0 &lt;= N &lt;= 100,000)에 있고, 동생은 점 K(0 &lt;= K &lt;= 100,000)에 있다.</t>
+          <t>1차원 BFS 동작 원리 및 개념 설명: 가중치가 1초로 동일한 상태 전이(X-1, X+1, 2*X)에서 최소 도달 시간을 구하기 위해 큐를 활용하여 가장 먼저 도달하는 시간을 기록하는 BFS 원리를 적용합니다.</t>
         </is>
       </c>
       <c r="N6" s="12" t="inlineStr">
@@ -8441,7 +8381,7 @@
       </c>
       <c r="J9" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>하준</t>
         </is>
       </c>
       <c r="K9" s="17" t="inlineStr">
@@ -8456,7 +8396,7 @@
       </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
-          <t>N×N 크기의 연구소에 바이러스가 유출되었다. 연구소의 각 칸은 빈 칸(0), 벽(1), 바이러스가 있는 칸(2) 중 하나이다.</t>
+          <t>생명공학 연구원 하준이는 연구실 격자 배양기에서 특정 바이러스가 확산되는 시간을 관찰하고 있다. N×N 크기의 연구소에 바이러스가 유출되었다.</t>
         </is>
       </c>
       <c r="N9" s="17" t="inlineStr">
@@ -8511,7 +8451,7 @@
       </c>
       <c r="J10" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>도윤</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -8526,7 +8466,7 @@
       </c>
       <c r="M10" s="12" t="inlineStr">
         <is>
-          <t>어떤 지역의 높이 정보를 파악하여, 많은 비가 내렸을 때 물에 잠기지 않는 안전한 영역이 최대 몇 개가 만들어지는지 조사하려고 한다. 지역은 N×N 크기의 2차원 배열로 표현되며 각 칸의 값은 해당 지점의 높이를 나...</t>
+          <t>기상 분석관 도윤이는 집중호우가 내렸을 때 침수되지 않고 물 위에 안전하게 남는 지대들의 개수를 조사하고 있다. 어떤 지역의 높이 정보를 파악하여, 많은 비가 내렸을 때 물에 잠기지 않는 안전한 영역이 최대 몇 개가...</t>
         </is>
       </c>
       <c r="N10" s="12" t="inlineStr">
@@ -8581,7 +8521,7 @@
       </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>시우</t>
         </is>
       </c>
       <c r="K11" s="17" t="inlineStr">
@@ -8596,7 +8536,7 @@
       </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>격자 모양 상자들을 수직으로 쌓아 올려 토마토를 보관하는 3차원 창고가 있다. 창고의 가로 칸 수 M, 세로 칸 수 N, 쌓아올려진 상자의 수 H가 주어진다.</t>
+          <t>스마트팜 창고를 관리하는 시우는 보관 중인 토마토들이 익은 토마토의 영향을 받아 모두 익는 데 걸리는 최소 일수를 계산하고자 한다. 격자 모양 상자들을 수직으로 쌓아 올려 토마토를 보관하는 3차원 창고가 있다.</t>
         </is>
       </c>
       <c r="N11" s="17" t="inlineStr">
@@ -9156,7 +9096,7 @@
       </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>정사각형 모양의 N×N 지도에 아파트들이 1로 표시되어 있다. 0은 집이 없는 빈 곳이다. 상, 하, 좌, 우로 연결된 집들의 모임을 하나의 '단지'라고 정의한다.</t>
+          <t>깊이 우선 탐색(DFS) 알고리즘 개념 및 동작 원리 설명: 깊이 우선 탐색(DFS)은 2차원 격자에서 인접한 연결 요소를 끝까지 파고들며 방문 배열을 통해 이미 센 집을 중복 방문하지 않고 묶어내는 영역 분할 알고...</t>
         </is>
       </c>
       <c r="N19" s="17" t="inlineStr">
@@ -9226,7 +9166,7 @@
       </c>
       <c r="M20" s="12" t="inlineStr">
         <is>
-          <t>신종 바이러스인 웜 바이러스는 네트워크를 통해 전파된다. 어느 날 1번 컴퓨터가 웜 바이러스에 걸렸다.</t>
+          <t>그래프 DFS 순회 개념 및 동작 원리 설명: 인접 리스트로 표현된 네트워크 그래프에서 1번 노드부터 재귀 호출을 통해 연결된 모든 노드를 완전 탐색하며 방문 노드 수를 누적하는 DFS 원리입니다.</t>
         </is>
       </c>
       <c r="N20" s="12" t="inlineStr">
@@ -9366,7 +9306,7 @@
       </c>
       <c r="M22" s="12" t="inlineStr">
         <is>
-          <t>N×M 크기의 2차원 격자 지도가 있다. 지도에서 1은 땅을 나타내고, 0은 바다를 나타낸다.</t>
+          <t>격자 그래프 연결 요소(Connected Component) 탐색 원리 및 개념 설명: 격자의 모든 좌표를 순회하며 아직 방문하지 않은 육지(1)를 발견할 때마다 DFS 재귀 호출을 시작하여 하나의 독립된 섬을 완전...</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -9421,7 +9361,7 @@
       </c>
       <c r="J23" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서준</t>
         </is>
       </c>
       <c r="K23" s="17" t="inlineStr">
@@ -9436,7 +9376,7 @@
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 격자 미로가 주어진다. 미로에서 0은 빈 통로, 1은 벽이다.</t>
+          <t>국립공원 탐방로 설계자 서준이는 등산객들이 출발지에서 도착지까지 안전하게 이동할 수 있는 유효 경로의 총 개수를 집계하고 있다. N×M 크기의 격자 미로가 주어진다.</t>
         </is>
       </c>
       <c r="N23" s="17" t="inlineStr">
@@ -9561,7 +9501,7 @@
       </c>
       <c r="J25" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>은우</t>
         </is>
       </c>
       <c r="K25" s="17" t="inlineStr">
@@ -9576,7 +9516,7 @@
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>세로 R칸, 가로 C칸으로 된 체스판 모양의 보드가 있다. 보드의 각 칸에는 대문자 알파벳이 하나씩 적혀 있고, 좌상단 (1행, 1열)에 말이 놓여 있다.</t>
+          <t>보드게임 개발자 은우는 동일한 알파벳을 중복해서 밟지 않으면서 보드판을 최대한 멀리 여행하는 말판 이동 규칙을 만들었다. 세로 R칸, 가로 C칸으로 된 체스판 모양의 보드가 있다.</t>
         </is>
       </c>
       <c r="N25" s="17" t="inlineStr">
@@ -9631,7 +9571,7 @@
       </c>
       <c r="J26" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유준</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
@@ -9646,7 +9586,7 @@
       </c>
       <c r="M26" s="12" t="inlineStr">
         <is>
-          <t>통로의 크기가 N×M인 건물이 있다. 통로의 곳곳에 음식물 쓰레기가 떨어져 있다.</t>
+          <t>캠핑장 청소 당번 유준이는 야영장 바닥에 떨어진 음식물 쓰레기들이 인접하여 형성하는 가장 큰 덩어리의 크기를 조사하여 청소 계획을 세우고 있다. 통로의 크기가 N×M인 건물이 있다.</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -9701,7 +9641,7 @@
       </c>
       <c r="J27" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>선우</t>
         </is>
       </c>
       <c r="K27" s="17" t="inlineStr">
@@ -9716,7 +9656,7 @@
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 모눈종이 위에 치즈가 놓여 있다. 치즈는 1로, 공기는 0으로 표시된다. 모눈종이의 맨 가장자리는 항상 치즈가 놓이지 않는 외부 공기이다.</t>
+          <t>식품 보관 연구원 선우는 냉장 창고의 외부 공기와 맞닿은 치즈 표면이 시간에 따라 서서히 녹아내리는 과정을 시뮬레이션하고 있다. N×M 크기의 모눈종이 위에 치즈가 놓여 있다.</t>
         </is>
       </c>
       <c r="N27" s="17" t="inlineStr">
@@ -10791,7 +10731,7 @@
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>이서의_01_배낭_최대_가치</t>
+          <t>이서의_동전_교환_최소_동전수</t>
         </is>
       </c>
       <c r="E43" s="13" t="inlineStr">
@@ -10826,7 +10766,7 @@
       </c>
       <c r="K43" s="17" t="inlineStr">
         <is>
-          <t>DP/D3_DP_이서의_01_배낭_최대_가치</t>
+          <t>DP/D3_DP_이서의_동전_교환_최소_동전수</t>
         </is>
       </c>
       <c r="L43" s="15" t="inlineStr">
@@ -10836,7 +10776,7 @@
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>고고학 발굴 탐사 대장인 이서는 유적지에서 귀중한 보물 N개를 발견했습니다. 각 보물 i는 무게 W_i와 가치 V_i를 지니고 있습니다.</t>
+          <t>스마트 자판기 프로젝트를 진행하는 이서는 거스름돈 반환 모듈을 설계하고 있습니다. N가지 서로 다른 가치를 가진 동전들이 무제한으로 주어질 때, 고객에게 K원의 거스름돈을 거슬러 주기 위해 필요한 최소 동전의 개수를...</t>
         </is>
       </c>
       <c r="N43" s="17" t="inlineStr">
@@ -11141,7 +11081,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>최장_증가_부분수열_LIS</t>
+          <t>파일_합치기_최소_비용</t>
         </is>
       </c>
       <c r="E48" s="13" t="inlineStr">
@@ -11176,7 +11116,7 @@
       </c>
       <c r="K48" s="12" t="inlineStr">
         <is>
-          <t>DP/D4_DP_최장_증가_부분수열_LIS</t>
+          <t>DP/D4_DP_파일_합치기_최소_비용</t>
         </is>
       </c>
       <c r="L48" s="10" t="inlineStr">
@@ -11186,7 +11126,7 @@
       </c>
       <c r="M48" s="12" t="inlineStr">
         <is>
-          <t>크기가 N인 수열 A가 주어질 때, 원소들이 엄격하게 증가하는 부분 수열(Strictly Increasing Subsequence) 중 '가장 길이가 긴 수열'의 길이를 구해야 합니다. 1. 단순 DP로 O(N^2)...</t>
+          <t>소설의 여러 장(Chapter)이 각각 독립된 파일로 나누어져 있습니다. 두 개의 연속된 파일을 합쳐 하나의 임시 파일로 만들고, 이 임시 파일들을 다시 합치는 과정을 반복하여 최종 하나의 완성본 파일로 묶으려 합니...</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -11746,7 +11686,7 @@
       </c>
       <c r="M56" s="12" t="inlineStr">
         <is>
-          <t>도하는 남해안의 N개의 유인도 섬들을 연륙교(다리)로 모두 연결하는 프로젝트를 총괄하고 있습니다. 각 다리를 놓을 수 있는 해상 구간과 건설 비용이 주어집니다.</t>
+          <t>남해안에 흩어져 있는 유인도 섬들을 연륙교(다리)로 모두 연결하여 육로 통행이 가능하도록 망을 구축하는 국토 개발 프로젝트입니다. 모든 섬을 직·간접적으로 연결하면서 총 건설 비용을 최소화해야 합니다. • 핵심 알고...</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -11886,7 +11826,7 @@
       </c>
       <c r="M58" s="12" t="inlineStr">
         <is>
-          <t>통신망 설계 엔지니어인 이서는 N개의 통신 기지국을 초고속 광케이블로 상호 연결하는 국책 통신망을 구축하고자 합니다. 기지국 간에 광케이블을 포설할 수 있는 구간 M개와 포설 비용이 주어집니다.</t>
+          <t>도시 인프라 설계를 담당하는 이서는 N개 연구 단지를 초고속 광케이블로 상호 연결하는 통신망을 구축하고자 합니다. 통신 지연을 최소화하면서 케이블 매설 비용의 총합을 최소화해야 합니다. • 핵심 알고리즘: 최소 신장...</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -11956,7 +11896,7 @@
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>이준이는 국토교통부 신임 도시계획관으로 임명되어 N개의 주요 도시를 연결하는 고속도로망을 구축해야 합니다. 각 도시간 고속도로 건설 후보 구간 M개와 그에 따른 공사 비용이 주어집니다.</t>
+          <t>교통 시스템 연구원인 이준이는 전국 N개 물류 거점 도시들을 고속도로로 연결하는 국가 간선 도로망을 설계하고 있습니다. 모든 도시 간에 차량 이동이 가능하도록 연결하면서 총 도로 포장 비용을 최소화합니다. • 핵심 ...</t>
         </is>
       </c>
       <c r="N59" s="17" t="inlineStr">
@@ -12026,7 +11966,7 @@
       </c>
       <c r="M60" s="12" t="inlineStr">
         <is>
-          <t>수자원 공사의 엔지니어인 하윤이는 산간 지역 N개 마을에 깨끗한 수돗물을 공급하기 위한 파이프라인 매설 계획을 수립하고 있습니다. 마을 간 파이프 매설 가능 경로 M개와 공사 비용이 주어집니다.</t>
+          <t>스마트 시티 수자원 관리 엔지니어인 하윤이는 N개 신도시 단지에 깨끗한 수돗물을 공급하기 위해 상수도 파이프라인망을 구축하고 있습니다. 물이 고립되는 구역 없이 모든 단지에 급수가 이루어지도록 최소 비용 파이프라인을...</t>
         </is>
       </c>
       <c r="N60" s="12" t="inlineStr">
@@ -12096,7 +12036,7 @@
       </c>
       <c r="M61" s="17" t="inlineStr">
         <is>
-          <t>이미 N개의 정점으로 구성된 최소 신장 트리(MST)가 완성되어 있으며, 기존 트리의 가중치 합은 initialWeight입니다. 여기에 새로운 간선 (u, v, w) 하나가 추가 제안되었습니다.</t>
+          <t>기존에 완성된 최소 신장 트리(MST)에 새로운 간선 (u, v, w)가 추가되면 정확히 하나의 단순 사이클이 형성됩니다. 트리의 연결성을 유지하면서 가중치 합을 최소로 유지하기 위해, 형성된 사이클 상에서 가장 가...</t>
         </is>
       </c>
       <c r="N61" s="17" t="inlineStr">
@@ -12236,7 +12176,7 @@
       </c>
       <c r="M63" s="17" t="inlineStr">
         <is>
-          <t>최소 병목 스패닝 트리(Minimum Bottleneck Spanning Tree, MBST)는 그래프의 모든 정점을 연결하는 스패닝 트리 중, 포함된 간선들 중 '가장 가중치가 큰 간선의 가중치(Max Edge W...</t>
+          <t>스패닝 트리의 간선들 중 '가장 비용이 큰 단일 간선의 가중치(병목 비용)'를 최소화하는 트리(Min-Bottleneck Spanning Tree, MBST)를 구하는 문제입니다. 크루스칼 알고리즘으로 구한 MST의...</t>
         </is>
       </c>
       <c r="N63" s="17" t="inlineStr">
@@ -12376,7 +12316,7 @@
       </c>
       <c r="M65" s="17" t="inlineStr">
         <is>
-          <t>2차원 평면 위에 N개의 행성 기지가 위치해 있습니다. 각 기지의 좌표는 (x, y) 정수 좌표로 주어집니다. 모든 두 행성 기지 (i, j) 사이에는 우주 터널을 뚫을 수 있으며, 두 기지를 연결하는 터널의 건설 ...</t>
+          <t>2차원 평면 위에 N개의 통신 관측소 좌표 (x_i, y_i)가 주어집니다. 두 관측소 사이를 유선 케이블로 연결할 때의 비용은 두 점 사이의 유클리드 거리(또는 거리의 제곱에 비례)입니다. 모든 관측소를 하나의 통...</t>
         </is>
       </c>
       <c r="N65" s="17" t="inlineStr">
@@ -14476,7 +14416,7 @@
       </c>
       <c r="M95" s="17" t="inlineStr">
         <is>
-          <t>$R \times C$ 크기의 미로 격자판이 있습니다. 각 칸은 빈 칸(0)이거나, 부술 수 있는 특수 방화벽(1)입니다.</t>
+          <t>R x C 크기의 미로 격자판이 있습니다. 각 칸은 빈 칸(0)이거나, 부술 수 있는 특수 방화벽(1)입니다.</t>
         </is>
       </c>
       <c r="N95" s="17" t="inlineStr">
@@ -14616,7 +14556,7 @@
       </c>
       <c r="M97" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 정수 수열 A와 임계값 K가 주어집니다. 수열의 연속된 부분 구간 $[left, right]$에 대하여, 구간 내의 최댓값과 최솟값의 차이가 K 이하인 구간을 '안정 구간'이라고 부릅니다:</t>
+          <t>길이가 N인 정수 수열 A와 임계값 K가 주어집니다. 수열의 연속된 부분 구간 [left, right]에 대하여, 구간 내의 최댓값과 최솟값의 차이가 K 이하인 구간을 '안정 구간'이라고 부릅니다:</t>
         </is>
       </c>
       <c r="N97" s="17" t="inlineStr">
@@ -14811,7 +14751,7 @@
       </c>
       <c r="J100" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
@@ -14826,7 +14766,7 @@
       </c>
       <c r="M100" s="12" t="inlineStr">
         <is>
-          <t>SSAFY 검색 엔진 팀에서 텍스트 문서 T 내에서 검색 키워드 패턴 P가 총 몇 번 등장하는지, 그리고 가장 먼저 등장하는 시작 위치(1-based 인덱스)가 어디인지 빠르게 확인하는 기능을 구현하고자 합니다. 패...</t>
+          <t>도서관 정보 검색실의 로운이는 방대한 고문서 텍스트 속에서 특정 고유 패턴이 나타나는 모든 위치를 KMP 알고리즘으로 빠르게 검색하고 있다. SSAFY 검색 엔진 팀에서 텍스트 문서 T 내에서 검색 키워드 패턴 P가...</t>
         </is>
       </c>
       <c r="N100" s="12" t="inlineStr">
@@ -15301,7 +15241,7 @@
       </c>
       <c r="J107" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서아</t>
         </is>
       </c>
       <c r="K107" s="17" t="inlineStr">
@@ -15316,7 +15256,7 @@
       </c>
       <c r="M107" s="17" t="inlineStr">
         <is>
-          <t>1부터 9까지의 숫자가 사용되는 스도쿠에서, 특정 빈 칸과 같은 행, 같은 열, 같은 3x3 박스에 이미 사용된 숫자들의 집합이 주어집니다. 사용된 숫자 집합을 비트마스크(1&lt;&lt;숫자)로 표현하여 합집합을 구한 뒤, ...</t>
+          <t>퍼즐 동아리의 서아는 스도쿠 빈칸에 들어갈 수 있는 후보 숫자들을 비트마스크 부분집합으로 표현하여 유효성을 판별하고 있다. 1부터 9까지의 숫자가 사용되는 스도쿠에서, 특정 빈 칸과 같은 행, 같은 열, 같은 3x3...</t>
         </is>
       </c>
       <c r="N107" s="17" t="inlineStr">
@@ -15371,7 +15311,7 @@
       </c>
       <c r="J108" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아윤</t>
         </is>
       </c>
       <c r="K108" s="12" t="inlineStr">
@@ -15386,7 +15326,7 @@
       </c>
       <c r="M108" s="12" t="inlineStr">
         <is>
-          <t>N개의 자연수로 구성된 집합이 주어집니다. 이 집합을 두 개의 서로소 부분집합 A와 B로 나누어, 두 부분집합의 원소의 합이 정확히 같아질 수 있는지 판별하십시오.</t>
+          <t>보석 세공사 아윤이는 수집한 원석들을 두 개의 상자에 담을 때 두 상자의 총 가치가 정확히 같아지도록 부분집합을 분할하고자 한다. N개의 자연수로 구성된 집합이 주어집니다.</t>
         </is>
       </c>
       <c r="N108" s="12" t="inlineStr">
@@ -16156,7 +16096,7 @@
       </c>
       <c r="M119" s="17" t="inlineStr">
         <is>
-          <t>배열에서 최댓값과 최솟값을 동시에 찾을 때, 일반적인 반복문은 $2N - 2$번의 비교를 수행합니다. 하지만 분할 정복(Tournament 방식)을 사용하면 약 $3N/2 - 2$번의 비교만으로 최댓값과 최솟값을 동...</t>
+          <t>배열에서 최댓값과 최솟값을 동시에 찾을 때, 일반적인 반복문은 2N - 2번의 비교를 수행합니다. 하지만 분할 정복(Tournament 방식)을 사용하면 약 3N/2 - 2번의 비교만으로 최댓값과 최솟값을 동시에 찾...</t>
         </is>
       </c>
       <c r="N119" s="17" t="inlineStr">
@@ -16436,7 +16376,7 @@
       </c>
       <c r="M123" s="17" t="inlineStr">
         <is>
-          <t>선우는 물리 시뮬레이션 프로그램을 제작하던 중, 상태 전이 행렬 A를 B번 연속하여 곱해야 하는 상황에 직면했습니다. 행렬의 크기 M x M(2 &lt;= M &lt;= 5)과 지수 B(1 &lt;= B &lt;= 100,000,000,...</t>
+          <t>선우는 금융 데이터의 점화식 상태 전이를 고속으로 계산하기 위해 K x K 정방행렬 A의 N제곱(A^N)을 계산해야 합니다. N이 최대 10^12에 달하므로, 지수를 절반씩 나누어 계산하는 분할 정복 기법(A^N =...</t>
         </is>
       </c>
       <c r="N123" s="17" t="inlineStr">
@@ -16506,7 +16446,7 @@
       </c>
       <c r="M124" s="12" t="inlineStr">
         <is>
-          <t>아윤이는 흑백 영상을 효율적으로 압축하여 전송하는 쿼드 트리(Quad Tree) 알고리즘을 구현하고 있습니다. N x N 크기의 흑백 영상은 각 픽셀이 0(흰색) 또는 1(검은색)로 구성되어 있습니다. (N은 2의 ...</t>
+          <t>컴퓨터 그래픽스를 공부하는 아윤이는 흑백 영상(0과 1로 구성된 N x N 격자)을 압축하기 위해 쿼드트리(Quad Tree) 방식을 구현하고 있습니다. 영역 전체가 모두 같은 색이면 그 숫자로 압축하고, 그렇지 않...</t>
         </is>
       </c>
       <c r="N124" s="12" t="inlineStr">
@@ -16576,7 +16516,7 @@
       </c>
       <c r="M125" s="17" t="inlineStr">
         <is>
-          <t>유준이는 색종이 공예를 하기 위해 N x N 크기의 격자 종이를 가지고 있습니다. N은 3의 거듭제곱($3^k$, 1 &lt;= k &lt;= 7)입니다.</t>
+          <t>유준이는 N x N 크기의 색종이를 가지고 놀고 있습니다. 종이의 모든 칸이 -1, 0, 1 중 같은 숫자로 채워져 있지 않다면, 가로와 세로를 각각 3등분하여 총 9개의 동일한 크기의 작은 종이로 자르고 이 과정을...</t>
         </is>
       </c>
       <c r="N125" s="17" t="inlineStr">
@@ -16646,7 +16586,7 @@
       </c>
       <c r="M126" s="12" t="inlineStr">
         <is>
-          <t>지아는 자료구조 시간에 이진 트리의 전위 순회(Preorder)와 중위 순회(Inorder) 결과를 전달받았습니다. 트리를 구성하는 모든 노드는 1부터 N까지 서로 다른 고유한 자연수 번호를 가지고 있습니다.</t>
+          <t>자료구조를 연구하는 지아는 어떤 이진 트리를 전위 순회(Preorder)한 결과와 중위 순회(Inorder)한 결과를 전달받았습니다. 전위 순회의 첫 번째 원소가 항상 서브트리의 루트임을 이용하고, 중위 순회에서 루...</t>
         </is>
       </c>
       <c r="N126" s="12" t="inlineStr">
@@ -16786,7 +16726,7 @@
       </c>
       <c r="M128" s="12" t="inlineStr">
         <is>
-          <t>크기가 N인 정수 배열에서 K번째(1-based)로 작은 원소를 찾는 문제입니다. 전체 배열을 정렬하면 $O(N \log N)$이 걸리지만, 퀵소트(Quick Sort)의 분할 정복 기법을 변형한 퀵 셀렉트(Quic...</t>
+          <t>정렬되지 않은 N개의 데이터에서 K번째로 작은 원소를 정렬 없이 평균 O(N) 시간에 찾아내는 퀵셀렉트(Quickselect) 알고리즘입니다. 피벗(Pivot)을 기준으로 파티셔닝을 수행한 후, K의 위치가 속한 분...</t>
         </is>
       </c>
       <c r="N128" s="12" t="inlineStr">
@@ -16856,7 +16796,7 @@
       </c>
       <c r="M129" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 수열 A에서 $i &lt; j$이면서 $A[i] &gt; A[j]$인 쌍 $(i, j)$를 '역순쌍(Inversion)'이라고 합니다. 단순 이중 반복문으로 역순쌍을 셀 경우 $O(N^2)$ 시간이 걸려 $N=10...</t>
+          <t>크기 N인 배열 A에서 i &lt; j 이지만 A[i] &gt; A[j]를 만족하는 쌍 (i, j)를 역순쌍(Inversion)이라고 합니다. 단순 이중 루프 O(N^2)로는 100,000 크기의 배열을 처리할 수 없으므로, ...</t>
         </is>
       </c>
       <c r="N129" s="17" t="inlineStr">
@@ -16926,7 +16866,7 @@
       </c>
       <c r="M130" s="12" t="inlineStr">
         <is>
-          <t>길이가 N인 정수 배열 A에서 연속된 부분 배열(Subarray)의 합 중 최댓값을 구하는 문제입니다. (적어도 하나의 원소는 선택해야 합니다.) 이 문제는 대표적인 분할 정복(Divide and Conquer) 응...</t>
+          <t>연속된 부분 배열의 원소 합 중 최댓값을 구하는 문제입니다. 배열을 좌우 두 영역으로 나누어, 1) 왼쪽 영역의 최대 부분합, 2) 오른쪽 영역의 최대 부분합, 3) 중앙 경계를 가로지르는 최대 부분합을 각각 분할 ...</t>
         </is>
       </c>
       <c r="N130" s="12" t="inlineStr">
@@ -16996,7 +16936,7 @@
       </c>
       <c r="M131" s="17" t="inlineStr">
         <is>
-          <t>피보나치 수열은 $F_0 = 0, F_1 = 1$, 그리고 $N \ge 2$에 대해 $F_N = F_{N-1} + F_{N-2}$로 정의됩니다. $N$이 매우 클 때(최대 $10^{16}$), 동적 계획법(DP)으로...</t>
+          <t>피보나치 수열의 N번째 항 F_N을 구하는 문제입니다. N이 10^18까지 주어지므로 동적 계획법 O(N)으로도 해결할 수 없습니다. 상태 전이 행렬 [[1, 1], [1, 0]]의 N제곱을 분할 정복(Matrix ...</t>
         </is>
       </c>
       <c r="N131" s="17" t="inlineStr">
@@ -17696,7 +17636,7 @@
       </c>
       <c r="M141" s="17" t="inlineStr">
         <is>
-          <t>나은이는 정보 동아리에서 0부터 N까지 N+1개의 원소로 구성된 집합들을 관리하고 있습니다. 처음에는 모든 원소가 각각 하나의 집합을 이룹니다.</t>
+          <t>나은이는 1부터 N까지의 원소들로 구성된 서로소 집합 자료구조를 공부하고 있습니다. 두 원소가 속한 집합을 합치는 연산(0 a b)과, 두 원소가 같은 집합에 속해 있는지 확인하는 연산(1 a b)이 질의 형태로 주...</t>
         </is>
       </c>
       <c r="N141" s="17" t="inlineStr">
@@ -17906,7 +17846,7 @@
       </c>
       <c r="M144" s="12" t="inlineStr">
         <is>
-          <t>시아는 R x C 크기의 지도에서 바다(0)와 육지(1)를 관리하는 국토 개발 프로젝트를 진행하고 있습니다. 상하좌우로 인접한 육지(1)들은 하나의 섬을 형성합니다.</t>
+          <t>해양 탐험가 시아는 군도에 위치한 N개의 섬들 사이에 다리를 놓는 작업을 진행하고 있습니다. 다리가 하나씩 건설될 때마다 두 섬이 속한 군집이 합쳐집니다. 시아를 도와 각 연결 쿼리 후 현재 독립적인 연결 컴포넌트의...</t>
         </is>
       </c>
       <c r="N144" s="12" t="inlineStr">
@@ -17976,7 +17916,7 @@
       </c>
       <c r="M145" s="17" t="inlineStr">
         <is>
-          <t>아린이는 교내 여러 동아리들의 연합 규모를 조사하고 있습니다. 교내에는 1부터 N까지 번호가 붙은 N명의 학생이 있습니다.</t>
+          <t>학생회장 아린이는 교내 N명의 학생들이 구성하는 동아리 연합 네트워크를 분석하고 있습니다. 친구 관계인 두 학생은 같은 동아리로 묶이며, 친구의 친구 역시 동일한 동아리에 속합니다. 모든 관계가 주어졌을 때 가장 구...</t>
         </is>
       </c>
       <c r="N145" s="17" t="inlineStr">
@@ -18046,7 +17986,7 @@
       </c>
       <c r="M146" s="12" t="inlineStr">
         <is>
-          <t>가중치 유니온 파인드(Weighted Union-Find)는 각 원소 간의 상대적 차이(Potential Difference)를 추적할 수 있는 확장 자료구조입니다. 연구소에서 N개의 물건의 무게를 비교하고 있습니다...</t>
+          <t>각 정점 x, y 사이의 상대적 무게 차이(weight[y] - weight[x] = w)를 유지하고 질의하는 문제입니다. 경로 압축 시 루트와의 상대 오프셋(Potential)을 누적 갱신하여, 두 원소 간의 무게...</t>
         </is>
       </c>
       <c r="N146" s="12" t="inlineStr">
@@ -18186,7 +18126,7 @@
       </c>
       <c r="M148" s="12" t="inlineStr">
         <is>
-          <t>서로소 집합은 집합을 합치는(Union) 연산은 매우 빠르지만, 이미 합쳐진 집합을 쪼개거나 간선을 제거하는 연산은 직접 지원하지 않습니다. 따라서 간선이 시간 순서대로 제거되는 문제는 질의를 끝에서부터 거꾸로 역순...</t>
+          <t>그래프에서 간선이 하나씩 '제거'되는 상황에서의 연결성 질의는 일반적인 유니온파인드로 직접 처리하기 어렵습니다. 쿼리를 모두 수집한 뒤, 모든 간선이 제거된 최종 상태에서 역순(시간 역류)으로 간선을 '추가(Unio...</t>
         </is>
       </c>
       <c r="N148" s="12" t="inlineStr">
@@ -18256,7 +18196,7 @@
       </c>
       <c r="M149" s="17" t="inlineStr">
         <is>
-          <t>두 팀으로 나누어 시합을 하려고 합니다. 일부 참가자 쌍 사이에 '적대 관계'가 주어집니다.</t>
+          <t>정점 u와 v가 서로 다른 색으로 칠해져야 한다는 조건들이 동적으로 추가될 때, 그래프가 이분 그래프(Bipartite Graph)로 유지되는지 실시간으로 판별합니다. 각 원소 x에 대해 동치 관계 x와 반대 관계 ...</t>
         </is>
       </c>
       <c r="N149" s="17" t="inlineStr">
@@ -18326,7 +18266,7 @@
       </c>
       <c r="M150" s="12" t="inlineStr">
         <is>
-          <t>초기에 1부터 N까지 N개의 단독 노드로 이루어진 시스템이 있습니다. 네트워크 간선이 하나씩 순차적으로 추가될 때마다, 전체 네트워크에서 '가장 큰 연결 컴포넌트(Maximum Connected Component)의...</t>
+          <t>N개의 정점이 있는 무방향 그래프에서 간선이 하나씩 추가될 때마다, 전체 그래프에서 가장 원소 수가 많은 연결 컴포넌트의 크기(최댓값)를 즉각 반환하는 동적 질의 문제입니다. 각 집합의 크기를 루트 노드에 저장하고 ...</t>
         </is>
       </c>
       <c r="N150" s="12" t="inlineStr">
@@ -19011,7 +18951,7 @@
       </c>
       <c r="J160" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>지아</t>
         </is>
       </c>
       <c r="K160" s="12" t="inlineStr">
@@ -19026,7 +18966,7 @@
       </c>
       <c r="M160" s="12" t="inlineStr">
         <is>
-          <t>1부터 N까지의 숫자로 이루어진 순열이 주어졌을 때, 사전순으로 바로 다음에 오는 순열을 찾는 알고리즘을 구현합니다. 만약 이미 사전순으로 마지막 순열(내림차순)이라면 -1을 출력합니다.</t>
+          <t>보안 시스템 연구원 지아는 비밀번호 순열 목록에서 사전순으로 바로 다음에 오는 순열을 생성하는 인증 알고리즘을 개발 중이다. 1부터 N까지의 숫자로 이루어진 순열이 주어졌을 때, 사전순으로 바로 다음에 오는 순열을 ...</t>
         </is>
       </c>
       <c r="N160" s="12" t="inlineStr">
@@ -19151,7 +19091,7 @@
       </c>
       <c r="J162" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>하윤</t>
         </is>
       </c>
       <c r="K162" s="12" t="inlineStr">
@@ -19166,7 +19106,7 @@
       </c>
       <c r="M162" s="12" t="inlineStr">
         <is>
-          <t>N명의 사람(1번부터 N번)이 원형 테이블에 둘러앉습니다. 회전하여 일치하는 배치는 동일한 것으로 간주합니다.</t>
+          <t>연회 기획자 하윤이는 귀빈들을 원형 테이블에 둘러앉힐 때 서로 사이가 좋은 사람들끼리 이웃하도록 순열 좌석을 배치하고 있다. N명의 사람(1번부터 N번)이 원형 테이블에 둘러앉습니다.</t>
         </is>
       </c>
       <c r="N162" s="12" t="inlineStr">
@@ -19261,7 +19201,7 @@
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>과일트럭_최단배달</t>
+          <t>N자리_순열_사전순_K번째_복원</t>
         </is>
       </c>
       <c r="E164" s="13" t="inlineStr">
@@ -19296,7 +19236,7 @@
       </c>
       <c r="K164" s="12" t="inlineStr">
         <is>
-          <t>순열/D4_순열_과일트럭_최단배달</t>
+          <t>순열/D4_순열_N자리_순열_사전순_K번째_복원</t>
         </is>
       </c>
       <c r="L164" s="10" t="inlineStr">
@@ -19306,7 +19246,7 @@
       </c>
       <c r="M164" s="12" t="inlineStr">
         <is>
-          <t>신선 과일 배송 트럭이 과일 유통센터(0번)에서 출발하여 N개의 가맹 과일 매장(1번부터 N번)을 모두 정확히 한 번씩 방문하여 배송을 마친 뒤, 다시 유통센터(0번)로 복귀해야 합니다. 지점 i에서 지점 j로 이동...</t>
+          <t>1부터 N까지의 자연수를 한 번씩만 사용하여 만들 수 있는 N!개의 순열들을 사전순으로 정렬했을 때, K번째로 오는 순열을 복원하는 문제입니다. N이 최대 20에 달할 수 있으므로 N! = 2.4 x 10^18로 모...</t>
         </is>
       </c>
       <c r="N164" s="12" t="inlineStr">
@@ -19331,7 +19271,7 @@
       </c>
       <c r="D165" s="16" t="inlineStr">
         <is>
-          <t>부등호_관계식_최대_최소_수열</t>
+          <t>과일트럭_최단배달</t>
         </is>
       </c>
       <c r="E165" s="13" t="inlineStr">
@@ -19366,7 +19306,7 @@
       </c>
       <c r="K165" s="17" t="inlineStr">
         <is>
-          <t>순열/D4_순열_부등호_관계식_최대_최소_수열</t>
+          <t>순열/D4_순열_과일트럭_최단배달</t>
         </is>
       </c>
       <c r="L165" s="15" t="inlineStr">
@@ -19376,7 +19316,7 @@
       </c>
       <c r="M165" s="17" t="inlineStr">
         <is>
-          <t>주어진 부등호 관계식을 만족하는 k+1자리의 최대 정수와 최소 정수를 각각 문자열 형태로 한 줄씩 출력하십시오.</t>
+          <t>신선 과일 배송 트럭이 과일 유통센터(0번)에서 출발하여 N개의 가맹 과일 매장(1번부터 N번)을 모두 정확히 한 번씩 방문하여 배송을 마친 뒤, 다시 유통센터(0번)로 복귀해야 합니다. 지점 i에서 지점 j로 이동...</t>
         </is>
       </c>
       <c r="N165" s="17" t="inlineStr">
@@ -19401,7 +19341,7 @@
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>부등호_수열_생성</t>
+          <t>부등호_관계식_최대_최소_수열</t>
         </is>
       </c>
       <c r="E166" s="13" t="inlineStr">
@@ -19436,7 +19376,7 @@
       </c>
       <c r="K166" s="12" t="inlineStr">
         <is>
-          <t>순열/D4_순열_부등호_수열_생성</t>
+          <t>순열/D4_순열_부등호_관계식_최대_최소_수열</t>
         </is>
       </c>
       <c r="L166" s="10" t="inlineStr">
@@ -19446,7 +19386,7 @@
       </c>
       <c r="M166" s="12" t="inlineStr">
         <is>
-          <t>k개의 부등호 기호('&lt;', '&gt;')가 나열된 순열이 주어집니다. 0부터 9까지의 서로 다른 숫자 k+1개를 골라 부등호 관계를 모두 만족하도록 배치하여 k+1자리 정수를 만듭니다.</t>
+          <t>주어진 부등호 관계식을 만족하는 k+1자리의 최대 정수와 최소 정수를 각각 문자열 형태로 한 줄씩 출력하십시오.</t>
         </is>
       </c>
       <c r="N166" s="12" t="inlineStr">
@@ -20776,7 +20716,7 @@
       </c>
       <c r="M185" s="17" t="inlineStr">
         <is>
-          <t>알파벳 소문자로 구성된 긴 원본 문자열 S와 목표 단어 T가 주어집니다. S 안에서 길이 $|T|$인 연속된 부분 문자열 중, T의 문자들을 재배열하여 만들 수 있는 부분 문자열(아나그램, Anagram)이 몇 번 ...</t>
+          <t>알파벳 소문자로 구성된 긴 원본 문자열 S와 목표 단어 T가 주어집니다. S 안에서 길이 |T|인 연속된 부분 문자열 중, T의 문자들을 재배열하여 만들 수 있는 부분 문자열(아나그램, Anagram)이 몇 번 등장...</t>
         </is>
       </c>
       <c r="N185" s="17" t="inlineStr">
@@ -20816,7 +20756,7 @@
       </c>
       <c r="G186" s="10" t="inlineStr">
         <is>
-          <t>25985-V2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H186" s="12" t="inlineStr">
@@ -21476,7 +21416,7 @@
       </c>
       <c r="M195" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 수열 A와 윈도우 크기 L이 주어집니다. 수열에서 $i = 0$부터 $N - L$까지 각 윈도우 $[i, i + L - 1]$의 최솟값을 모두 구해야 합니다.</t>
+          <t>길이가 N인 수열 A와 윈도우 크기 L이 주어집니다. 수열에서 i = 0부터 N - L까지 각 윈도우 [i, i + L - 1]의 최솟값을 모두 구해야 합니다.</t>
         </is>
       </c>
       <c r="N195" s="17" t="inlineStr">
@@ -22036,7 +21976,7 @@
       </c>
       <c r="M203" s="17" t="inlineStr">
         <is>
-          <t>단일 연결 리스트에서 전체 크기를 미리 세지 않고도 정중앙의 노드를 단 한 번의 순회($O(N)$)로 찾아내는 대표적인 알고리즘이 바로 '투 포인터 러너(Runner) 기법'입니다. 두 개의 포인터 `slow`와 `...</t>
+          <t>단일 연결 리스트에서 전체 크기를 미리 세지 않고도 정중앙의 노드를 단 한 번의 순회(O(N))로 찾아내는 대표적인 알고리즘이 바로 '투 포인터 러너(Runner) 기법'입니다. 두 개의 포인터 `slow`와 `fa...</t>
         </is>
       </c>
       <c r="N203" s="17" t="inlineStr">
@@ -22736,7 +22676,7 @@
       </c>
       <c r="M213" s="17" t="inlineStr">
         <is>
-          <t>1번부터 N번까지의 사람이 원형으로 둘러앉아 있을 때, 순서대로 K번째 사람을 탈락시키는 요세푸스 순열 문제입니다. 일반적인 배열이나 단순 큐를 사용할 경우 $K$가 매우 크거나 노드 삭제가 빈번할 때 $O(N \t...</t>
+          <t>1번부터 N번까지의 사람이 원형으로 둘러앉아 있을 때, 순서대로 K번째 사람을 탈락시키는 요세푸스 순열 문제입니다. 일반적인 배열이나 단순 큐를 사용할 경우 K가 매우 크거나 노드 삭제가 빈번할 때 O(N x K)의...</t>
         </is>
       </c>
       <c r="N213" s="17" t="inlineStr">
@@ -23296,7 +23236,7 @@
       </c>
       <c r="M221" s="17" t="inlineStr">
         <is>
-          <t>프로게이머 서윤이는 실시간 전략 시뮬레이션 게임(RTS)에서 최고의 연구 빌드오더를 설계하고 있습니다. 게임 내에는 1번부터 N번까지 총 N개의 기술(Tech)이 존재합니다.</t>
+          <t>게임 개발자 서윤이는 전략 시뮬레이션 게임에서 건물이나 유닛을 생산하기 위한 테크트리 선행 관계를 정의하고 있습니다. 특정 기술을 연구하려면 선행 기술들이 모두 완료되어야 합니다. 주어진 선행 관계를 바탕으로 모든 ...</t>
         </is>
       </c>
       <c r="N221" s="17" t="inlineStr">
@@ -23366,7 +23306,7 @@
       </c>
       <c r="M222" s="12" t="inlineStr">
         <is>
-          <t>DJ 선우는 음악 스트리밍 파티를 위해 1번부터 N번까지 N곡으로 구성된 플레이리스트를 제작 중입니다. 선우는 곡의 분위기(BPM, Mood) 전개가 자연스럽도록 M개의 곡 순서 규칙을 정했습니다.</t>
+          <t>음악 스트리밍 DJ 선우는 청취자의 몰입도를 높이기 위해 곡 간의 자연스러운 흐름 선행 조건을 반영한 플레이리스트를 제작하려 합니다. 특정 곡 u는 반드시 곡 v보다 먼저 재생되어야 한다는 조건들을 모두 만족하는 유...</t>
         </is>
       </c>
       <c r="N222" s="12" t="inlineStr">
@@ -23436,7 +23376,7 @@
       </c>
       <c r="M223" s="17" t="inlineStr">
         <is>
-          <t>유주는 생일 선물로 거대한 로봇 레고 블록 키트를 선물 받았습니다. 키트에는 1번부터 N번까지의 부품들이 있으며, 설명서에는 M개의 선행 조립 관계(부품 u를 먼저 조립해야 부품 v를 결합할 수 있음)가 적혀 있습니...</t>
+          <t>조립 블록 마니아 유주는 N개의 부품으로 구성된 거대 로봇을 조립하고 있습니다. 특정 부품들은 다른 기본 부품들이 먼저 조립되어 결합되어야만 다음 조립이 가능합니다. 유주가 부품들을 올바른 순서대로 조립할 수 있도록...</t>
         </is>
       </c>
       <c r="N223" s="17" t="inlineStr">
@@ -23506,7 +23446,7 @@
       </c>
       <c r="M224" s="12" t="inlineStr">
         <is>
-          <t>소프트웨어 PM인 은우는 대규모 프로젝트의 스프린트 태스크들을 관리하고 있습니다. 프로젝트에는 1번부터 N번까지 N개의 단위 작업(Task)이 있으며, 작업 간의 의존 관계(Dependency) M개가 주어집니다.</t>
+          <t>프로젝트 매니저 은우는 소프트웨어 릴리스를 위해 N개의 하위 태스크를 계획하고 있습니다. 태스크 간의 선행 의존성(Dependency)을 해결하여 작업자들에게 순차적으로 배분할 수 있는 작업 실행 일정을 수립하십시오...</t>
         </is>
       </c>
       <c r="N224" s="12" t="inlineStr">
@@ -23576,7 +23516,7 @@
       </c>
       <c r="M225" s="17" t="inlineStr">
         <is>
-          <t>전략 시뮬레이션 게임에서 건물 1번부터 N번까지 각각을 짓는 데 걸리는 건설 시간 time[i]가 주어집니다. 또한 건물 간의 선행 건설 조건 M개가 주어집니다.</t>
+          <t>건물을 짓는 데 걸리는 시간 D_i와 건물 간의 선행 건설 규칙이 주어집니다. 여러 건물을 동시에 병렬로 지을 수 있을 때, 특정 목표 건물 W를 완성하기까지 걸리는 최소 총 소요 시간을 구하는 문제입니다. 진입 차...</t>
         </is>
       </c>
       <c r="N225" s="17" t="inlineStr">
@@ -23646,7 +23586,7 @@
       </c>
       <c r="M226" s="12" t="inlineStr">
         <is>
-          <t>방향 그래프가 주어졌을 때, 위상 정렬의 가능한 결과가 다음 세 가지 중 어느 것에 해당하는지 판별하는 문제입니다: 1. "CYCLE": 그래프에 사이클이 존재하여 위상 정렬이 불가능한 경우</t>
+          <t>주어진 방향 그래프의 위상 정렬 순서가 '유일하게 단 하나만 존재하는지(Unique)', '여러 가지 순서가 가능한지(Multiple)', 아니면 '사이클이 발생하여 불가능한지(Cycle)'를 판별하는 고난도 알고리...</t>
         </is>
       </c>
       <c r="N226" s="12" t="inlineStr">
@@ -23716,7 +23656,7 @@
       </c>
       <c r="M227" s="17" t="inlineStr">
         <is>
-          <t>민우는 1번부터 N번까지 총 N개의 문제로 구성된 문제집을 풀려고 합니다. 문제들은 난이도 순서대로 1번이 가장 쉽고 N번이 가장 어렵습니다.</t>
+          <t>N개의 문제를 풀어야 합니다. 문제 간에 먼저 풀어야 하는 선행 조건이 주어지고, 선행 조건이 없는 문제들 중에서는 번호가 작은 문제를 먼저 푸는 것이 좋습니다. 일반 큐 대신 최소 힙(Min-PriorityQueu...</t>
         </is>
       </c>
       <c r="N227" s="17" t="inlineStr">
@@ -23741,7 +23681,7 @@
       </c>
       <c r="D228" s="11" t="inlineStr">
         <is>
-          <t>임계_경로_최장_소요_시간</t>
+          <t>사전순_가장_앞선_위상정렬</t>
         </is>
       </c>
       <c r="E228" s="13" t="inlineStr">
@@ -23776,7 +23716,7 @@
       </c>
       <c r="K228" s="12" t="inlineStr">
         <is>
-          <t>위상정렬/D4_위상정렬_임계_경로_최장_소요_시간</t>
+          <t>위상정렬/D4_위상정렬_사전순_가장_앞선_위상정렬</t>
         </is>
       </c>
       <c r="L228" s="10" t="inlineStr">
@@ -23786,7 +23726,7 @@
       </c>
       <c r="M228" s="12" t="inlineStr">
         <is>
-          <t>임계 경로(Critical Path) 기법은 대규모 건설 및 소프트웨어 프로젝트에서 전체 작업이 완료되는 최단 완료 시간(즉, 선행 제약으로 인한 최장 경로의 길이)을 계산하는 핵심 알고리즘입니다. 프로젝트의 각 작...</t>
+          <t>N개의 문제로 구성된 알고리즘 문제집이 있습니다. 각 문제는 1번부터 N번까지 번호가 매겨져 있습니다. 문제들 사이에는 특정 문제를 다른 문제보다 먼저 푸는 것이 좋은 M개의 선행 규칙이 주어집니다.</t>
         </is>
       </c>
       <c r="N228" s="12" t="inlineStr">
@@ -23811,7 +23751,7 @@
       </c>
       <c r="D229" s="16" t="inlineStr">
         <is>
-          <t>임계경로_작업_스케줄러</t>
+          <t>임계_경로_최장_소요_시간</t>
         </is>
       </c>
       <c r="E229" s="13" t="inlineStr">
@@ -23846,7 +23786,7 @@
       </c>
       <c r="K229" s="17" t="inlineStr">
         <is>
-          <t>위상정렬/D4_위상정렬_임계경로_작업_스케줄러</t>
+          <t>위상정렬/D4_위상정렬_임계_경로_최장_소요_시간</t>
         </is>
       </c>
       <c r="L229" s="15" t="inlineStr">
@@ -23856,7 +23796,7 @@
       </c>
       <c r="M229" s="17" t="inlineStr">
         <is>
-          <t>대형 건설 프로젝트에는 1번부터 N번까지 총 N개의 작업이 있습니다. 각 작업 i는 완료하는 데 t_i 시간이 소요되며, 작업들 간의 선후 관계가 방향 비순환 그래프(DAG)로 주어집니다.</t>
+          <t>대규모 건설 프로젝트에서 전체 공정이 완료되는 최소 시간(즉, 시작점에서 도착점까지의 최장 경로)을 계산하고, 이 완료 시간에 직접적인 영향을 미치는 임계 경로 간선들의 총 개수를 역추적(Backtracking)하여...</t>
         </is>
       </c>
       <c r="N229" s="17" t="inlineStr">
@@ -24206,7 +24146,7 @@
       </c>
       <c r="M234" s="12" t="inlineStr">
         <is>
-          <t>이진 탐색(Binary Search) 알고리즘 개념 및 동작 원리 설명: 이진 탐색은 '오름차순으로 정렬된 배열'에서 특정 목표 값(Target)의 위치를 $O(\log N)$ 시간 복잡도로 빠르게 찾아내는 탐색 알...</t>
+          <t>이진 탐색(Binary Search) 알고리즘 개념 및 동작 원리 설명: 이진 탐색은 '오름차순으로 정렬된 배열'에서 특정 목표 값(Target)의 위치를 O(log N) 시간 복잡도로 빠르게 찾아내는 탐색 알고리즘...</t>
         </is>
       </c>
       <c r="N234" s="12" t="inlineStr">
@@ -24556,7 +24496,7 @@
       </c>
       <c r="M239" s="17" t="inlineStr">
         <is>
-          <t>시우는 동아리 방의 네트워크를 재구축하기 위해 길이가 제각각인 K개의 랜선을 가지고 있습니다. 시우는 이 K개의 랜선을 잘라서 모두 같은 길이의 랜선 N개를 만들어야 합니다.</t>
+          <t>시우는 길이가 제각각인 K개의 랜선을 가지고 있습니다. 이 랜선들을 잘라서 모두 같은 길이의 랜선 N개를 만들고자 합니다. 자른 후 남은 랜선 조각은 버려집니다. 만들 수 있는 최대 랜선 길이를 이진 탐색(Upper...</t>
         </is>
       </c>
       <c r="N239" s="17" t="inlineStr">
@@ -24626,7 +24566,7 @@
       </c>
       <c r="M240" s="12" t="inlineStr">
         <is>
-          <t>은우는 목공 실습 시간에 필요한 목재 M미터를 구하기 위해 숲으로 갔습니다. 숲에는 일렬로 심어진 N그루의 나무가 있으며, 각 나무의 높이가 주어집니다.</t>
+          <t>은우는 목재 공장에서 벌목 작업을 하고 있습니다. N개의 나무들이 한 줄로 서 있고, 절단기의 높이를 H로 지정하면 H보다 높은 나무들의 윗부분이 잘려 나갑니다. 은우가 필요한 최소 M미터의 나무를 가져가기 위해 설...</t>
         </is>
       </c>
       <c r="N240" s="12" t="inlineStr">
@@ -24696,7 +24636,7 @@
       </c>
       <c r="M241" s="17" t="inlineStr">
         <is>
-          <t>국가 예산 관리자인 하윤이는 여러 지방 부처의 예산 요청을 심사하여 국가 총예산 범위 내에서 배정하려고 합니다. 각 부처는 필요한 예산 요청액을 제출했습니다.</t>
+          <t>재정 담당관 하윤이는 N개 지자체의 예산 요청을 심사하여 국가 총예산 M원 내에서 배정하고자 합니다. 모든 요청의 총합이 M 이하이면 요청한 금액을 그대로 배정하고, 초과하면 특정 상한액(Cap)을 정하여 상한액 이...</t>
         </is>
       </c>
       <c r="N241" s="17" t="inlineStr">
@@ -24766,7 +24706,7 @@
       </c>
       <c r="M242" s="12" t="inlineStr">
         <is>
-          <t>크기가 N x N인 2차원 배열 A가 있습니다. 배열의 각 행과 열은 1부터 시작하며, A[i][j] = i * j 입니다. 이 수를 1차원 배열 B에 모두 넣으면 크기가 N^2인 배열이 됩니다.</t>
+          <t>N x N 크기의 2차원 배열 A의 각 원소는 A[i][j] = i * j 입니다. 이 수들을 1차원 배열 B에 넣고 오름차순 정렬했을 때, B[K]번째에 위치하는 수를 구하는 문제입니다. N이 최대 10^5로 N^...</t>
         </is>
       </c>
       <c r="N242" s="12" t="inlineStr">
@@ -24976,7 +24916,7 @@
       </c>
       <c r="M245" s="17" t="inlineStr">
         <is>
-          <t>보석 상자에 M가지 서로 다른 색상의 보석이 들어 있습니다. i번째 색상의 보석은 count[i]개 존재합니다.</t>
+          <t>M가지 색상의 보석들이 각각 몇 개씩 주어지고, N명의 학생들에게 보석을 나누어 주려고 합니다. 각 학생은 한 가지 색상의 보석만 받을 수 있으며, 받지 못하는 학생이 있어도 됩니다. 가장 많은 보석을 받은 학생이 ...</t>
         </is>
       </c>
       <c r="N245" s="17" t="inlineStr">
@@ -25046,7 +24986,7 @@
       </c>
       <c r="M246" s="12" t="inlineStr">
         <is>
-          <t>국제공항 입국심사대에서 N명의 심사관이 대기 중인 M명의 승객을 심사하려고 합니다. 각 심사관마다 한 명의 승객을 심사하는 데 걸리는 시간(times[i])이 제각기 다릅니다.</t>
+          <t>입국 심사대 N개가 있고 각 심사관마다 한 사람을 심사하는 데 걸리는 시간 T_k가 다릅니다. 심사를 기다리는 입국자 M명이 있을 때, 모든 사람이 심사를 완료하는 데 걸리는 최소 총 소요 시간을 구하십시오. 시간 ...</t>
         </is>
       </c>
       <c r="N246" s="12" t="inlineStr">
@@ -25326,7 +25266,7 @@
       </c>
       <c r="M250" s="12" t="inlineStr">
         <is>
-          <t>자연수 N이 주어졌을 때, 각 자릿수의 합을 재귀적으로 구하는 함수 `digitSum(n)`을 작성합니다: - 기저 조건: $N &lt; 10$이면 $N$을 반환</t>
+          <t>자연수 N이 주어졌을 때, 각 자릿수의 합을 재귀적으로 구하는 함수 `digitSum(n)`을 작성합니다: - 기저 조건: N &lt; 10이면 N을 반환</t>
         </is>
       </c>
       <c r="N250" s="12" t="inlineStr">
@@ -25536,7 +25476,7 @@
       </c>
       <c r="M253" s="17" t="inlineStr">
         <is>
-          <t>자연수 C와 N이 주어질 때, $C^N$을 재귀 호출을 이용하여 계산하는 문제입니다. 기저 조건: $N = 0$일 때 결과는 1입니다.</t>
+          <t>자연수 C와 N이 주어질 때, C^N을 재귀 호출을 이용하여 계산하는 문제입니다. 기저 조건: N = 0일 때 결과는 1입니다.</t>
         </is>
       </c>
       <c r="N253" s="17" t="inlineStr">
@@ -25886,7 +25826,7 @@
       </c>
       <c r="M258" s="12" t="inlineStr">
         <is>
-          <t>초등학생 이준이는 장난감 사각 블록을 가지고 프랙탈 카펫 패턴을 조립하고 있습니다. $3^K \times 3^K$ 크기의 정사각형 판에서, 정중앙의 $3^{K-1} \times 3^{K-1}$ 영역은 블록을 비워두고...</t>
+          <t>초등학생 이준이는 장난감 사각 블록을 가지고 프랙탈 카펫 패턴을 조립하고 있습니다. 3^K x 3^K 크기의 정사각형 판에서, 정중앙의 3^{K-1} x 3^{K-1} 영역은 블록을 비워두고, 나머지 8개의 영역은 ...</t>
         </is>
       </c>
       <c r="N258" s="12" t="inlineStr">
@@ -26026,7 +25966,7 @@
       </c>
       <c r="M260" s="12" t="inlineStr">
         <is>
-          <t>한 변의 길이가 $2^N$인 2차원 배열을 'Z' 모양으로 재귀 탐색합니다. $2 \times 2$ 배열에서는 왼쪽 위(0) -&gt; 오른쪽 위(1) -&gt; 왼쪽 아래(2) -&gt; 오른쪽 아래(3) 순서로 방문합니다.</t>
+          <t>한 변의 길이가 2^N인 2차원 배열을 'Z' 모양으로 재귀 탐색합니다. 2 x 2 배열에서는 왼쪽 위(0) -&gt; 오른쪽 위(1) -&gt; 왼쪽 아래(2) -&gt; 오른쪽 아래(3) 순서로 방문합니다.</t>
         </is>
       </c>
       <c r="N260" s="12" t="inlineStr">
@@ -26096,7 +26036,7 @@
       </c>
       <c r="M261" s="17" t="inlineStr">
         <is>
-          <t>크기 $3^K \times 3^K$의 시에르핀스키 카펫 격자를 재귀적으로 생성하는 문제입니다. $K=1$인 경우 가운데 한 칸이 공백이고 주변 8칸이 별('*')인 패턴입니다:</t>
+          <t>크기 3^K x 3^K의 시에르핀스키 카펫 격자를 재귀적으로 생성하는 문제입니다. K=1인 경우 가운데 한 칸이 공백이고 주변 8칸이 별('*')인 패턴입니다:</t>
         </is>
       </c>
       <c r="N261" s="17" t="inlineStr">
@@ -26166,7 +26106,7 @@
       </c>
       <c r="M262" s="12" t="inlineStr">
         <is>
-          <t>$N \times N$ ($N = 2^K$) 크기의 흑백 영상이 주어집니다. 각 픽셀은 흰색(0) 또는 검은색(1)입니다. 쿼드 트리(Quad Tree) 알고리즘을 사용하여 영상을 다음과 같이 재귀적으로 압축합니다:</t>
+          <t>N x N (N = 2^K) 크기의 흑백 영상이 주어집니다. 각 픽셀은 흰색(0) 또는 검은색(1)입니다. 쿼드 트리(Quad Tree) 알고리즘을 사용하여 영상을 다음과 같이 재귀적으로 압축합니다:</t>
         </is>
       </c>
       <c r="N262" s="12" t="inlineStr">
@@ -26306,7 +26246,7 @@
       </c>
       <c r="M264" s="12" t="inlineStr">
         <is>
-          <t>세 개의 기둥(1번, 2번, 3번)과 크기가 서로 다른 N개의 원판이 1번 기둥에 꽂혀 있습니다. 하노이의 탑 규칙에 따라 모든 원판을 3번 기둥으로 옮기려면 총 $2^N - 1$번의 이동이 필요합니다.</t>
+          <t>세 개의 기둥(1번, 2번, 3번)과 크기가 서로 다른 N개의 원판이 1번 기둥에 꽂혀 있습니다. 하노이의 탑 규칙에 따라 모든 원판을 3번 기둥으로 옮기려면 총 2^N - 1번의 이동이 필요합니다.</t>
         </is>
       </c>
       <c r="N264" s="12" t="inlineStr">
@@ -26991,7 +26931,7 @@
       </c>
       <c r="J274" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서윤</t>
         </is>
       </c>
       <c r="K274" s="12" t="inlineStr">
@@ -27006,7 +26946,7 @@
       </c>
       <c r="M274" s="12" t="inlineStr">
         <is>
-          <t>짝수 N명의 사람이 모여 축구 시합을 하려고 합니다. N명을 정확히 N/2명씩 스타트 팀과 링크 팀으로 나눕니다. 사람 i와 j가 같은 팀에 속했을 때 팀에 더해지는 시너지 능력치 S_ij가 2차원 배열로 주어집니다...</t>
+          <t>체육대회 운영위원 서윤이는 전체 인원을 두 팀으로 공평하게 나눌 때 팀 간의 능력치 차이가 최소가 되는 최적의 조합을 찾고 있다. 짝수 N명의 사람이 모여 축구 시합을 하려고 합니다. N명을 정확히 N/2명씩 스타트...</t>
         </is>
       </c>
       <c r="N274" s="12" t="inlineStr">
@@ -27061,7 +27001,7 @@
       </c>
       <c r="J275" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="K275" s="17" t="inlineStr">
@@ -27076,7 +27016,7 @@
       </c>
       <c r="M275" s="17" t="inlineStr">
         <is>
-          <t>과일 명품관에서 N가지 과일(1번부터 N번) 중 서로 다른 R개를 골라 고급 선물 바구니를 구성하려고 합니다 (순서 무관). 그런데 과일 전문가들의 연구에 따르면, 함께 담았을 때 숙성 가스나 향의 충돌로 맛을 해치...</t>
+          <t>수제 디저트 카페를 운영하는 시아는 매장의 대표 디저트 메뉴 중 조화로운 조합을 선택하여 한정판 선물 세트를 구성하려 한다. 과일 명품관에서 N가지 과일(1번부터 N번) 중 서로 다른 R개를 골라 고급 선물 바구니를...</t>
         </is>
       </c>
       <c r="N275" s="17" t="inlineStr">
@@ -27131,7 +27071,7 @@
       </c>
       <c r="J276" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아린</t>
         </is>
       </c>
       <c r="K276" s="12" t="inlineStr">
@@ -27146,7 +27086,7 @@
       </c>
       <c r="M276" s="12" t="inlineStr">
         <is>
-          <t>1부터 N까지의 자연수 중 서로 다른 6개의 수를 뽑아 로또 번호 조합을 만듭니다. 이때 '행운의 조건'으로 홀수의 개수가 정확히 3개(짝수도 3개)이고, 6개 수의 총합이 S 이상이어야 합니다.</t>
+          <t>통계학 연구원 아린이는 추첨 번호 후보군 중에서 수학적 확률 조건에 맞는 행운의 번호 조합들을 체계적으로 추출하고 있다. 1부터 N까지의 자연수 중 서로 다른 6개의 수를 뽑아 로또 번호 조합을 만듭니다.</t>
         </is>
       </c>
       <c r="N276" s="12" t="inlineStr">
@@ -27451,7 +27391,7 @@
       </c>
       <c r="D281" s="16" t="inlineStr">
         <is>
-          <t>스타트와_링크_팀_밸런스_최적화</t>
+          <t>도심_스프링클러_최적_감시_배치</t>
         </is>
       </c>
       <c r="E281" s="13" t="inlineStr">
@@ -27486,7 +27426,7 @@
       </c>
       <c r="K281" s="17" t="inlineStr">
         <is>
-          <t>조합/D4_조합_스타트와_링크_팀_밸런스_최적화</t>
+          <t>조합/D4_조합_도심_스프링클러_최적_감시_배치</t>
         </is>
       </c>
       <c r="L281" s="15" t="inlineStr">
@@ -27496,7 +27436,7 @@
       </c>
       <c r="M281" s="17" t="inlineStr">
         <is>
-          <t>주어진 능력치 행렬 S에 대해 스타트 팀과 링크 팀의 능력치 차이의 최솟값을 구하십시오.</t>
+          <t>도시 방재 본부에서는 N x N 크기의 도심 구역에서 화재 위험이 있는 잔디/건물 구역 H곳을 보호하기 위해, K개의 후보 위치 중 정확히 M개의 자동 스프링클러를 설치하려고 합니다. 각 보호 구역 h와 스프링클러 ...</t>
         </is>
       </c>
       <c r="N281" s="17" t="inlineStr">
@@ -27521,7 +27461,7 @@
       </c>
       <c r="D282" s="11" t="inlineStr">
         <is>
-          <t>치킨_배달_거리_최적화</t>
+          <t>스타트와_링크_팀_밸런스_최적화</t>
         </is>
       </c>
       <c r="E282" s="13" t="inlineStr">
@@ -27556,7 +27496,7 @@
       </c>
       <c r="K282" s="12" t="inlineStr">
         <is>
-          <t>조합/D4_조합_치킨_배달_거리_최적화</t>
+          <t>조합/D4_조합_스타트와_링크_팀_밸런스_최적화</t>
         </is>
       </c>
       <c r="L282" s="10" t="inlineStr">
@@ -27566,7 +27506,7 @@
       </c>
       <c r="M282" s="12" t="inlineStr">
         <is>
-          <t>주어진 도시 지도에서 치킨집 최대 M개를 남겼을 때 얻을 수 있는 도시의 최소 치킨 거리를 구하십시오.</t>
+          <t>주어진 능력치 행렬 S에 대해 스타트 팀과 링크 팀의 능력치 차이의 최솟값을 구하십시오.</t>
         </is>
       </c>
       <c r="N282" s="12" t="inlineStr">
@@ -27591,7 +27531,7 @@
       </c>
       <c r="D283" s="16" t="inlineStr">
         <is>
-          <t>치킨거리_최소화</t>
+          <t>치킨_배달_거리_최적화</t>
         </is>
       </c>
       <c r="E283" s="13" t="inlineStr">
@@ -27626,7 +27566,7 @@
       </c>
       <c r="K283" s="17" t="inlineStr">
         <is>
-          <t>조합/D4_조합_치킨거리_최소화</t>
+          <t>조합/D4_조합_치킨_배달_거리_최적화</t>
         </is>
       </c>
       <c r="L283" s="15" t="inlineStr">
@@ -27636,7 +27576,7 @@
       </c>
       <c r="M283" s="17" t="inlineStr">
         <is>
-          <t>N x N 크기의 도시에 집(1)과 치킨집(2)이 있습니다. 도시의 치킨집 중 최대 M개만을 남기고 나머지는 폐업시키려 합니다.</t>
+          <t>주어진 도시 지도에서 치킨집 최대 M개를 남겼을 때 얻을 수 있는 도시의 최소 치킨 거리를 구하십시오.</t>
         </is>
       </c>
       <c r="N283" s="17" t="inlineStr">
@@ -28041,7 +27981,7 @@
       </c>
       <c r="J289" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="K289" s="17" t="inlineStr">
@@ -28056,7 +27996,7 @@
       </c>
       <c r="M289" s="17" t="inlineStr">
         <is>
-          <t>탕후루 가게에서 N가지 과일(1번부터 N번)을 중복을 허용하여 꼬치에 아래에서부터 차례로 K개를 꽂아 만듭니다. 첫 입부터 마지막 입까지 씹히는 과일의 순서가 중요합니다.</t>
+          <t>축제 부스를 맡은 나은이는 여러 종류의 과일을 중복을 허용하여 꼬치에 꽂아 다채로운 맛의 탕후루 순서를 만들고 있다. 탕후루 가게에서 N가지 과일(1번부터 N번)을 중복을 허용하여 꼬치에 아래에서부터 차례로 K개를 ...</t>
         </is>
       </c>
       <c r="N289" s="17" t="inlineStr">
@@ -28181,7 +28121,7 @@
       </c>
       <c r="J291" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유주</t>
         </is>
       </c>
       <c r="K291" s="17" t="inlineStr">
@@ -28196,7 +28136,7 @@
       </c>
       <c r="M291" s="17" t="inlineStr">
         <is>
-          <t>신호등에는 R(빨강), G(초록), B(파랑) 3가지 색이 있습니다. K초 동안 매 초마다 한 가지 색을 켜는데, 에너지 효율을 위해 동일한 색이 연속으로 점등될 수 없습니다.</t>
+          <t>교통 안전 모니터링을 담당하는 유주는 교차로 신호등의 불빛 점등 신호 패턴을 중복순열 조합으로 분석하고 있다. 신호등에는 R(빨강), G(초록), B(파랑) 3가지 색이 있습니다.</t>
         </is>
       </c>
       <c r="N291" s="17" t="inlineStr">
@@ -28321,7 +28261,7 @@
       </c>
       <c r="J293" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이준</t>
         </is>
       </c>
       <c r="K293" s="17" t="inlineStr">
@@ -28336,7 +28276,7 @@
       </c>
       <c r="M293" s="17" t="inlineStr">
         <is>
-          <t>1부터 M까지의 눈금이 있는 M면체 주사위를 K번 던집니다 (중복 허용, 던지는 순서 있음). K번 던져 나온 모든 눈금의 합이 정확히 S가 되는 서로 다른 주사위 던지기 결과의 총수를 구하시오.</t>
+          <t>보드게임 제작자 이준이는 N개의 주사위를 굴렸을 때 나올 수 있는 모든 눈금의 순서쌍 중 특정 합을 만족하는 경우의 수를 집계하고 있다. 1부터 M까지의 눈금이 있는 M면체 주사위를 K번 던집니다 (중복 허용, 던지...</t>
         </is>
       </c>
       <c r="N293" s="17" t="inlineStr">
@@ -29231,7 +29171,7 @@
       </c>
       <c r="J306" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>도하</t>
         </is>
       </c>
       <c r="K306" s="12" t="inlineStr">
@@ -29246,7 +29186,7 @@
       </c>
       <c r="M306" s="12" t="inlineStr">
         <is>
-          <t>방정식 x_1 + x_2 + ... + x_N = K 를 만족하는 정수해의 개수를 구합니다. 단, 각 변수 x_i는 최소 L 이상이어야 합니다 (x_i &gt;= L).</t>
+          <t>수학 퀴즈 동아리의 도하는 음이 아닌 정수해를 구하는 연립 방정식 문제를 중복조합 원리로 풀어내는 프로그램을 작성하고 있다. 방정식 x_1 + x_2 + ... + x_N = K 를 만족하는 정수해의 개수를 구합니다...</t>
         </is>
       </c>
       <c r="N306" s="12" t="inlineStr">
@@ -29301,7 +29241,7 @@
       </c>
       <c r="J307" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이서</t>
         </is>
       </c>
       <c r="K307" s="17" t="inlineStr">
@@ -29316,7 +29256,7 @@
       </c>
       <c r="M307" s="17" t="inlineStr">
         <is>
-          <t>1부터 N까지의 자연수 중 중복을 허용하여 K개를 골라 비내림차순(a_1 &lt;= a_2 &lt;= ... &lt;= a_K) 수열을 만듭니다. 이 수열들 중 모든 원소의 합이 짝수인 수열의 총 개수를 구하시오.</t>
+          <t>음악 작곡가 이서는 피아노 건반의 음높이가 점점 낮아지지 않는 아름다운 멜로디 수열을 중복조합 원리로 생성하고 있다. 1부터 N까지의 자연수 중 중복을 허용하여 K개를 골라 비내림차순(a_1 &lt;= a_2 &lt;= ......</t>
         </is>
       </c>
       <c r="N307" s="17" t="inlineStr">
@@ -30531,7 +30471,7 @@
       </c>
       <c r="D325" s="16" t="inlineStr">
         <is>
-          <t>벨만포드_음수_사이클_검출</t>
+          <t>다익스트라_최단경로_역추적_복원</t>
         </is>
       </c>
       <c r="E325" s="13" t="inlineStr">
@@ -30566,7 +30506,7 @@
       </c>
       <c r="K325" s="17" t="inlineStr">
         <is>
-          <t>최단경로/D4_최단경로_벨만포드_음수_사이클_검출</t>
+          <t>최단경로/D4_최단경로_다익스트라_최단경로_역추적_복원</t>
         </is>
       </c>
       <c r="L325" s="15" t="inlineStr">
@@ -30576,7 +30516,7 @@
       </c>
       <c r="M325" s="17" t="inlineStr">
         <is>
-          <t>1번 도시에서 출발하여 도달 가능한 음수 사이클이 있으면 -1을 출력하고, 없으면 2번부터 N번 도시까지의 최단 거리를 한 줄에 하나씩 출력하십시오.</t>
+          <t>N개의 도시와 도시 사이를 잇는 M개의 일방통행 유료 버스 노선이 있습니다. 출발 도시 S에서 도착 도시 E까지 이동하는 최소 비용을 계산하고, 그 최소 비용을 달성하는 실제 최단 경로 상의 방문 도시 순서를 역추적...</t>
         </is>
       </c>
       <c r="N325" s="17" t="inlineStr">
@@ -30601,7 +30541,7 @@
       </c>
       <c r="D326" s="11" t="inlineStr">
         <is>
-          <t>벨만포드_타임머신_탐색</t>
+          <t>벨만포드_음수_사이클_검출</t>
         </is>
       </c>
       <c r="E326" s="13" t="inlineStr">
@@ -30636,7 +30576,7 @@
       </c>
       <c r="K326" s="12" t="inlineStr">
         <is>
-          <t>최단경로/D4_최단경로_벨만포드_타임머신_탐색</t>
+          <t>최단경로/D4_최단경로_벨만포드_음수_사이클_검출</t>
         </is>
       </c>
       <c r="L326" s="10" t="inlineStr">
@@ -30646,7 +30586,7 @@
       </c>
       <c r="M326" s="12" t="inlineStr">
         <is>
-          <t>N개의 도시가 있고, 도시 사이를 이동하는 M개의 버스 노선이 있습니다. 각 버스 노선은 출발 도시 u, 도착 도시 v, 그리고 이동 시간 w를 갖습니다.</t>
+          <t>1번 도시에서 출발하여 도달 가능한 음수 사이클이 있으면 -1을 출력하고, 없으면 2번부터 N번 도시까지의 최단 거리를 한 줄에 하나씩 출력하십시오.</t>
         </is>
       </c>
       <c r="N326" s="12" t="inlineStr">
@@ -31791,7 +31731,7 @@
       </c>
       <c r="D343" s="16" t="inlineStr">
         <is>
-          <t>이중_우선순위_큐_커스텀_구현</t>
+          <t>우선순위큐_중앙값_실시간_추적</t>
         </is>
       </c>
       <c r="E343" s="13" t="inlineStr">
@@ -31826,7 +31766,7 @@
       </c>
       <c r="K343" s="17" t="inlineStr">
         <is>
-          <t>큐/D4_큐_이중_우선순위_큐_커스텀_구현</t>
+          <t>큐/D4_큐_우선순위큐_중앙값_실시간_추적</t>
         </is>
       </c>
       <c r="L343" s="15" t="inlineStr">
@@ -31836,7 +31776,7 @@
       </c>
       <c r="M343" s="17" t="inlineStr">
         <is>
-          <t>주어진 N개의 연산을 모두 수행한 후, 큐가 비어있으면 "EMPTY"를 출력하고, 비어있지 않다면 최댓값과 최솟값을 공백으로 구분하여 출력하십시오.</t>
+          <t>빅데이터 스트리밍 관제 시스템에서 정수 데이터가 실시간으로 하나씩 순차 입력됩니다. 수가 하나씩 추가될 때마다 지금까지 입력된 수들 중 '중앙값(Median)'을 즉시 계산해야 합니다.</t>
         </is>
       </c>
       <c r="N343" s="17" t="inlineStr">
@@ -31861,7 +31801,7 @@
       </c>
       <c r="D344" s="11" t="inlineStr">
         <is>
-          <t>트럭의_다리_건너기</t>
+          <t>이중_우선순위_큐_커스텀_구현</t>
         </is>
       </c>
       <c r="E344" s="13" t="inlineStr">
@@ -31896,7 +31836,7 @@
       </c>
       <c r="K344" s="12" t="inlineStr">
         <is>
-          <t>큐/D4_큐_트럭의_다리_건너기</t>
+          <t>큐/D4_큐_이중_우선순위_큐_커스텀_구현</t>
         </is>
       </c>
       <c r="L344" s="10" t="inlineStr">
@@ -31906,7 +31846,7 @@
       </c>
       <c r="M344" s="12" t="inlineStr">
         <is>
-          <t>길이가 W이고 최대 하중 L까지 견딜 수 있는 일차선 다리가 있습니다. N대의 트럭이 정해진 순서대로 다리를 건너려고 합니다. 각 트럭의 무게는 A_1, A_2, ..., A_N입니다.</t>
+          <t>주어진 N개의 연산을 모두 수행한 후, 큐가 비어있으면 "EMPTY"를 출력하고, 비어있지 않다면 최댓값과 최솟값을 공백으로 구분하여 출력하십시오.</t>
         </is>
       </c>
       <c r="N344" s="12" t="inlineStr">
@@ -32046,7 +31986,7 @@
       </c>
       <c r="M346" s="12" t="inlineStr">
         <is>
-          <t>중복되지 않는 N개의 자연수로 이루어진 수열과 자연수 X가 주어집니다. 수열에서 서로 다른 두 원소 $A[i]$와 $A[j]$ ($i &lt; j$)를 골라 $A[i] + A[j] = X$를 만족하는 쌍의 총 개수를 구하...</t>
+          <t>중복되지 않는 N개의 자연수로 이루어진 수열과 자연수 X가 주어집니다. 수열에서 서로 다른 두 원소 A[i]와 A[j] (i &lt; j)를 골라 A[i] + A[j] = X를 만족하는 쌍의 총 개수를 구하는 문제입니다.</t>
         </is>
       </c>
       <c r="N346" s="12" t="inlineStr">
@@ -32256,7 +32196,7 @@
       </c>
       <c r="M349" s="17" t="inlineStr">
         <is>
-          <t>오름차순으로 정렬된 N개의 정수 수열과 목표값 Target이 주어집니다. 배열의 양 끝에서 시작하는 투 포인터를 조작하여, 두 수의 합이 Target이 되는 첫 번째 쌍 $(A[left], A[right])$을 찾아...</t>
+          <t>오름차순으로 정렬된 N개의 정수 수열과 목표값 Target이 주어집니다. 배열의 양 끝에서 시작하는 투 포인터를 조작하여, 두 수의 합이 Target이 되는 첫 번째 쌍 (A[left], A[right])을 찾아 두...</t>
         </is>
       </c>
       <c r="N349" s="17" t="inlineStr">
@@ -33121,7 +33061,7 @@
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 격자 미로가 주어진다. 미로에서 1은 이동할 수 있는 칸을 나타내고, 0은 이동할 수 없는 벽을 나타낸다.</t>
+          <t>너비 우선 탐색(BFS) 알고리즘 개념 및 동작 원리 설명: 너비 우선 탐색(BFS)은 시작 위치에서 출발하여 거리가 1인 칸부터 큐(Queue)에 넣어 가까운 곳부터 차례대로 탐색하는 대표적인 최단 경로 탐색 원리...</t>
         </is>
       </c>
     </row>
@@ -33241,7 +33181,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>수빈이는 동생과 숨바꼭질을 하고 있다. 수빈이는 현재 점 N(0 &lt;= N &lt;= 100,000)에 있고, 동생은 점 K(0 &lt;= K &lt;= 100,000)에 있다.</t>
+          <t>1차원 BFS 동작 원리 및 개념 설명: 가중치가 1초로 동일한 상태 전이(X-1, X+1, 2*X)에서 최소 도달 시간을 구하기 위해 큐를 활용하여 가장 먼저 도달하는 시간을 기록하는 BFS 원리를 적용합니다.</t>
         </is>
       </c>
     </row>
@@ -33321,7 +33261,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>정사각형 모양의 N×N 지도에 아파트들이 1로 표시되어 있다. 0은 집이 없는 빈 곳이다. 상, 하, 좌, 우로 연결된 집들의 모임을 하나의 '단지'라고 정의한다.</t>
+          <t>깊이 우선 탐색(DFS) 알고리즘 개념 및 동작 원리 설명: 깊이 우선 탐색(DFS)은 2차원 격자에서 인접한 연결 요소를 끝까지 파고들며 방문 배열을 통해 이미 센 집을 중복 방문하지 않고 묶어내는 영역 분할 알고...</t>
         </is>
       </c>
     </row>
@@ -33361,7 +33301,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>신종 바이러스인 웜 바이러스는 네트워크를 통해 전파된다. 어느 날 1번 컴퓨터가 웜 바이러스에 걸렸다.</t>
+          <t>그래프 DFS 순회 개념 및 동작 원리 설명: 인접 리스트로 표현된 네트워크 그래프에서 1번 노드부터 재귀 호출을 통해 연결된 모든 노드를 완전 탐색하며 방문 노드 수를 누적하는 DFS 원리입니다.</t>
         </is>
       </c>
     </row>
@@ -33441,7 +33381,7 @@
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 2차원 격자 지도가 있다. 지도에서 1은 땅을 나타내고, 0은 바다를 나타낸다.</t>
+          <t>격자 그래프 연결 요소(Connected Component) 탐색 원리 및 개념 설명: 격자의 모든 좌표를 순회하며 아직 방문하지 않은 육지(1)를 발견할 때마다 DFS 재귀 호출을 시작하여 하나의 독립된 섬을 완전...</t>
         </is>
       </c>
     </row>
@@ -34601,7 +34541,7 @@
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>배열에서 최댓값과 최솟값을 동시에 찾을 때, 일반적인 반복문은 $2N - 2$번의 비교를 수행합니다. 하지만 분할 정복(Tournament 방식)을 사용하면 약 $3N/2 - 2$번의 비교만으로 최댓값과 최솟값을 동...</t>
+          <t>배열에서 최댓값과 최솟값을 동시에 찾을 때, 일반적인 반복문은 2N - 2번의 비교를 수행합니다. 하지만 분할 정복(Tournament 방식)을 사용하면 약 3N/2 - 2번의 비교만으로 최댓값과 최솟값을 동시에 찾...</t>
         </is>
       </c>
     </row>
@@ -35481,7 +35421,7 @@
       </c>
       <c r="H62" s="12" t="inlineStr">
         <is>
-          <t>알파벳 소문자로 구성된 긴 원본 문자열 S와 목표 단어 T가 주어집니다. S 안에서 길이 $|T|$인 연속된 부분 문자열 중, T의 문자들을 재배열하여 만들 수 있는 부분 문자열(아나그램, Anagram)이 몇 번 ...</t>
+          <t>알파벳 소문자로 구성된 긴 원본 문자열 S와 목표 단어 T가 주어집니다. S 안에서 길이 |T|인 연속된 부분 문자열 중, T의 문자들을 재배열하여 만들 수 있는 부분 문자열(아나그램, Anagram)이 몇 번 등장...</t>
         </is>
       </c>
     </row>
@@ -35801,7 +35741,7 @@
       </c>
       <c r="H70" s="12" t="inlineStr">
         <is>
-          <t>단일 연결 리스트에서 전체 크기를 미리 세지 않고도 정중앙의 노드를 단 한 번의 순회($O(N)$)로 찾아내는 대표적인 알고리즘이 바로 '투 포인터 러너(Runner) 기법'입니다. 두 개의 포인터 `slow`와 `...</t>
+          <t>단일 연결 리스트에서 전체 크기를 미리 세지 않고도 정중앙의 노드를 단 한 번의 순회(O(N))로 찾아내는 대표적인 알고리즘이 바로 '투 포인터 러너(Runner) 기법'입니다. 두 개의 포인터 `slow`와 `fa...</t>
         </is>
       </c>
     </row>
@@ -36241,7 +36181,7 @@
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>이진 탐색(Binary Search) 알고리즘 개념 및 동작 원리 설명: 이진 탐색은 '오름차순으로 정렬된 배열'에서 특정 목표 값(Target)의 위치를 $O(\log N)$ 시간 복잡도로 빠르게 찾아내는 탐색 알...</t>
+          <t>이진 탐색(Binary Search) 알고리즘 개념 및 동작 원리 설명: 이진 탐색은 '오름차순으로 정렬된 배열'에서 특정 목표 값(Target)의 위치를 O(log N) 시간 복잡도로 빠르게 찾아내는 탐색 알고리즘...</t>
         </is>
       </c>
     </row>
@@ -36401,7 +36341,7 @@
       </c>
       <c r="H85" s="17" t="inlineStr">
         <is>
-          <t>자연수 N이 주어졌을 때, 각 자릿수의 합을 재귀적으로 구하는 함수 `digitSum(n)`을 작성합니다: - 기저 조건: $N &lt; 10$이면 $N$을 반환</t>
+          <t>자연수 N이 주어졌을 때, 각 자릿수의 합을 재귀적으로 구하는 함수 `digitSum(n)`을 작성합니다: - 기저 조건: N &lt; 10이면 N을 반환</t>
         </is>
       </c>
     </row>
@@ -36521,7 +36461,7 @@
       </c>
       <c r="H88" s="12" t="inlineStr">
         <is>
-          <t>자연수 C와 N이 주어질 때, $C^N$을 재귀 호출을 이용하여 계산하는 문제입니다. 기저 조건: $N = 0$일 때 결과는 1입니다.</t>
+          <t>자연수 C와 N이 주어질 때, C^N을 재귀 호출을 이용하여 계산하는 문제입니다. 기저 조건: N = 0일 때 결과는 1입니다.</t>
         </is>
       </c>
     </row>
@@ -37721,7 +37661,7 @@
       </c>
       <c r="H118" s="12" t="inlineStr">
         <is>
-          <t>중복되지 않는 N개의 자연수로 이루어진 수열과 자연수 X가 주어집니다. 수열에서 서로 다른 두 원소 $A[i]$와 $A[j]$ ($i &lt; j$)를 골라 $A[i] + A[j] = X$를 만족하는 쌍의 총 개수를 구하...</t>
+          <t>중복되지 않는 N개의 자연수로 이루어진 수열과 자연수 X가 주어집니다. 수열에서 서로 다른 두 원소 A[i]와 A[j] (i &lt; j)를 골라 A[i] + A[j] = X를 만족하는 쌍의 총 개수를 구하는 문제입니다.</t>
         </is>
       </c>
     </row>
@@ -37841,7 +37781,7 @@
       </c>
       <c r="H121" s="17" t="inlineStr">
         <is>
-          <t>오름차순으로 정렬된 N개의 정수 수열과 목표값 Target이 주어집니다. 배열의 양 끝에서 시작하는 투 포인터를 조작하여, 두 수의 합이 Target이 되는 첫 번째 쌍 $(A[left], A[right])$을 찾아...</t>
+          <t>오름차순으로 정렬된 N개의 정수 수열과 목표값 Target이 주어집니다. 배열의 양 끝에서 시작하는 투 포인터를 조작하여, 두 수의 합이 Target이 되는 첫 번째 쌍 (A[left], A[right])을 찾아 두...</t>
         </is>
       </c>
     </row>
@@ -38027,12 +37967,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>하준</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -38062,7 +38002,7 @@
       </c>
       <c r="I4" s="12" t="inlineStr">
         <is>
-          <t>N×N 크기의 연구소에 바이러스가 유출되었다. 연구소의 각 칸은 빈 칸(0), 벽(1), 바이러스가 있는 칸(2) 중 하나이다.</t>
+          <t>생명공학 연구원 하준이는 연구실 격자 배양기에서 특정 바이러스가 확산되는 시간을 관찰하고 있다. N×N 크기의 연구소에 바이러스가 유출되었다.</t>
         </is>
       </c>
     </row>
@@ -38072,12 +38012,12 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>도윤</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -38107,7 +38047,7 @@
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>어떤 지역의 높이 정보를 파악하여, 많은 비가 내렸을 때 물에 잠기지 않는 안전한 영역이 최대 몇 개가 만들어지는지 조사하려고 한다. 지역은 N×N 크기의 2차원 배열로 표현되며 각 칸의 값은 해당 지점의 높이를 나...</t>
+          <t>기상 분석관 도윤이는 집중호우가 내렸을 때 침수되지 않고 물 위에 안전하게 남는 지대들의 개수를 조사하고 있다. 어떤 지역의 높이 정보를 파악하여, 많은 비가 내렸을 때 물에 잠기지 않는 안전한 영역이 최대 몇 개가...</t>
         </is>
       </c>
     </row>
@@ -38117,12 +38057,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>시우</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -38152,7 +38092,7 @@
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>격자 모양 상자들을 수직으로 쌓아 올려 토마토를 보관하는 3차원 창고가 있다. 창고의 가로 칸 수 M, 세로 칸 수 N, 쌓아올려진 상자의 수 H가 주어진다.</t>
+          <t>스마트팜 창고를 관리하는 시우는 보관 중인 토마토들이 익은 토마토의 영향을 받아 모두 익는 데 걸리는 최소 일수를 계산하고자 한다. 격자 모양 상자들을 수직으로 쌓아 올려 토마토를 보관하는 3차원 창고가 있다.</t>
         </is>
       </c>
     </row>
@@ -38162,12 +38102,12 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서준</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -38197,7 +38137,7 @@
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 격자 미로가 주어진다. 미로에서 0은 빈 통로, 1은 벽이다.</t>
+          <t>국립공원 탐방로 설계자 서준이는 등산객들이 출발지에서 도착지까지 안전하게 이동할 수 있는 유효 경로의 총 개수를 집계하고 있다. N×M 크기의 격자 미로가 주어진다.</t>
         </is>
       </c>
     </row>
@@ -38252,12 +38192,12 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>은우</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -38287,7 +38227,7 @@
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>세로 R칸, 가로 C칸으로 된 체스판 모양의 보드가 있다. 보드의 각 칸에는 대문자 알파벳이 하나씩 적혀 있고, 좌상단 (1행, 1열)에 말이 놓여 있다.</t>
+          <t>보드게임 개발자 은우는 동일한 알파벳을 중복해서 밟지 않으면서 보드판을 최대한 멀리 여행하는 말판 이동 규칙을 만들었다. 세로 R칸, 가로 C칸으로 된 체스판 모양의 보드가 있다.</t>
         </is>
       </c>
     </row>
@@ -38297,12 +38237,12 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유준</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -38332,7 +38272,7 @@
       </c>
       <c r="I10" s="12" t="inlineStr">
         <is>
-          <t>통로의 크기가 N×M인 건물이 있다. 통로의 곳곳에 음식물 쓰레기가 떨어져 있다.</t>
+          <t>캠핑장 청소 당번 유준이는 야영장 바닥에 떨어진 음식물 쓰레기들이 인접하여 형성하는 가장 큰 덩어리의 크기를 조사하여 청소 계획을 세우고 있다. 통로의 크기가 N×M인 건물이 있다.</t>
         </is>
       </c>
     </row>
@@ -38342,12 +38282,12 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>선우</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
@@ -38377,7 +38317,7 @@
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>N×M 크기의 모눈종이 위에 치즈가 놓여 있다. 치즈는 1로, 공기는 0으로 표시된다. 모눈종이의 맨 가장자리는 항상 치즈가 놓이지 않는 외부 공기이다.</t>
+          <t>식품 보관 연구원 선우는 냉장 창고의 외부 공기와 맞닿은 치즈 표면이 시간에 따라 서서히 녹아내리는 과정을 시뮬레이션하고 있다. N×M 크기의 모눈종이 위에 치즈가 놓여 있다.</t>
         </is>
       </c>
     </row>
@@ -38537,7 +38477,7 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>이서의_01_배낭_최대_가치</t>
+          <t>이서의_동전_교환_최소_동전수</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
@@ -38552,12 +38492,12 @@
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>DP/D3_DP_이서의_01_배낭_최대_가치</t>
+          <t>DP/D3_DP_이서의_동전_교환_최소_동전수</t>
         </is>
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>고고학 발굴 탐사 대장인 이서는 유적지에서 귀중한 보물 N개를 발견했습니다. 각 보물 i는 무게 W_i와 가치 V_i를 지니고 있습니다.</t>
+          <t>스마트 자판기 프로젝트를 진행하는 이서는 거스름돈 반환 모듈을 설계하고 있습니다. N가지 서로 다른 가치를 가진 동전들이 무제한으로 주어질 때, 고객에게 K원의 거스름돈을 거슬러 주기 위해 필요한 최소 동전의 개수를...</t>
         </is>
       </c>
     </row>
@@ -38647,7 +38587,7 @@
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>도하는 남해안의 N개의 유인도 섬들을 연륙교(다리)로 모두 연결하는 프로젝트를 총괄하고 있습니다. 각 다리를 놓을 수 있는 해상 구간과 건설 비용이 주어집니다.</t>
+          <t>남해안에 흩어져 있는 유인도 섬들을 연륙교(다리)로 모두 연결하여 육로 통행이 가능하도록 망을 구축하는 국토 개발 프로젝트입니다. 모든 섬을 직·간접적으로 연결하면서 총 건설 비용을 최소화해야 합니다. • 핵심 알고...</t>
         </is>
       </c>
     </row>
@@ -38737,7 +38677,7 @@
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>통신망 설계 엔지니어인 이서는 N개의 통신 기지국을 초고속 광케이블로 상호 연결하는 국책 통신망을 구축하고자 합니다. 기지국 간에 광케이블을 포설할 수 있는 구간 M개와 포설 비용이 주어집니다.</t>
+          <t>도시 인프라 설계를 담당하는 이서는 N개 연구 단지를 초고속 광케이블로 상호 연결하는 통신망을 구축하고자 합니다. 통신 지연을 최소화하면서 케이블 매설 비용의 총합을 최소화해야 합니다. • 핵심 알고리즘: 최소 신장...</t>
         </is>
       </c>
     </row>
@@ -38782,7 +38722,7 @@
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>이준이는 국토교통부 신임 도시계획관으로 임명되어 N개의 주요 도시를 연결하는 고속도로망을 구축해야 합니다. 각 도시간 고속도로 건설 후보 구간 M개와 그에 따른 공사 비용이 주어집니다.</t>
+          <t>교통 시스템 연구원인 이준이는 전국 N개 물류 거점 도시들을 고속도로로 연결하는 국가 간선 도로망을 설계하고 있습니다. 모든 도시 간에 차량 이동이 가능하도록 연결하면서 총 도로 포장 비용을 최소화합니다. • 핵심 ...</t>
         </is>
       </c>
     </row>
@@ -38827,7 +38767,7 @@
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>수자원 공사의 엔지니어인 하윤이는 산간 지역 N개 마을에 깨끗한 수돗물을 공급하기 위한 파이프라인 매설 계획을 수립하고 있습니다. 마을 간 파이프 매설 가능 경로 M개와 공사 비용이 주어집니다.</t>
+          <t>스마트 시티 수자원 관리 엔지니어인 하윤이는 N개 신도시 단지에 깨끗한 수돗물을 공급하기 위해 상수도 파이프라인망을 구축하고 있습니다. 물이 고립되는 구역 없이 모든 단지에 급수가 이루어지도록 최소 비용 파이프라인을...</t>
         </is>
       </c>
     </row>
@@ -39287,12 +39227,12 @@
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -39322,7 +39262,7 @@
       </c>
       <c r="I32" s="12" t="inlineStr">
         <is>
-          <t>SSAFY 검색 엔진 팀에서 텍스트 문서 T 내에서 검색 키워드 패턴 P가 총 몇 번 등장하는지, 그리고 가장 먼저 등장하는 시작 위치(1-based 인덱스)가 어디인지 빠르게 확인하는 기능을 구현하고자 합니다. 패...</t>
+          <t>도서관 정보 검색실의 로운이는 방대한 고문서 텍스트 속에서 특정 고유 패턴이 나타나는 모든 위치를 KMP 알고리즘으로 빠르게 검색하고 있다. SSAFY 검색 엔진 팀에서 텍스트 문서 T 내에서 검색 키워드 패턴 P가...</t>
         </is>
       </c>
     </row>
@@ -39377,12 +39317,12 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서아</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -39412,7 +39352,7 @@
       </c>
       <c r="I34" s="12" t="inlineStr">
         <is>
-          <t>1부터 9까지의 숫자가 사용되는 스도쿠에서, 특정 빈 칸과 같은 행, 같은 열, 같은 3x3 박스에 이미 사용된 숫자들의 집합이 주어집니다. 사용된 숫자 집합을 비트마스크(1&lt;&lt;숫자)로 표현하여 합집합을 구한 뒤, ...</t>
+          <t>퍼즐 동아리의 서아는 스도쿠 빈칸에 들어갈 수 있는 후보 숫자들을 비트마스크 부분집합으로 표현하여 유효성을 판별하고 있다. 1부터 9까지의 숫자가 사용되는 스도쿠에서, 특정 빈 칸과 같은 행, 같은 열, 같은 3x3...</t>
         </is>
       </c>
     </row>
@@ -39422,12 +39362,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아윤</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
@@ -39457,7 +39397,7 @@
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>N개의 자연수로 구성된 집합이 주어집니다. 이 집합을 두 개의 서로소 부분집합 A와 B로 나누어, 두 부분집합의 원소의 합이 정확히 같아질 수 있는지 판별하십시오.</t>
+          <t>보석 세공사 아윤이는 수집한 원석들을 두 개의 상자에 담을 때 두 상자의 총 가치가 정확히 같아지도록 부분집합을 분할하고자 한다. N개의 자연수로 구성된 집합이 주어집니다.</t>
         </is>
       </c>
     </row>
@@ -39592,7 +39532,7 @@
       </c>
       <c r="I38" s="12" t="inlineStr">
         <is>
-          <t>선우는 물리 시뮬레이션 프로그램을 제작하던 중, 상태 전이 행렬 A를 B번 연속하여 곱해야 하는 상황에 직면했습니다. 행렬의 크기 M x M(2 &lt;= M &lt;= 5)과 지수 B(1 &lt;= B &lt;= 100,000,000,...</t>
+          <t>선우는 금융 데이터의 점화식 상태 전이를 고속으로 계산하기 위해 K x K 정방행렬 A의 N제곱(A^N)을 계산해야 합니다. N이 최대 10^12에 달하므로, 지수를 절반씩 나누어 계산하는 분할 정복 기법(A^N =...</t>
         </is>
       </c>
     </row>
@@ -39637,7 +39577,7 @@
       </c>
       <c r="I39" s="17" t="inlineStr">
         <is>
-          <t>아윤이는 흑백 영상을 효율적으로 압축하여 전송하는 쿼드 트리(Quad Tree) 알고리즘을 구현하고 있습니다. N x N 크기의 흑백 영상은 각 픽셀이 0(흰색) 또는 1(검은색)로 구성되어 있습니다. (N은 2의 ...</t>
+          <t>컴퓨터 그래픽스를 공부하는 아윤이는 흑백 영상(0과 1로 구성된 N x N 격자)을 압축하기 위해 쿼드트리(Quad Tree) 방식을 구현하고 있습니다. 영역 전체가 모두 같은 색이면 그 숫자로 압축하고, 그렇지 않...</t>
         </is>
       </c>
     </row>
@@ -39682,7 +39622,7 @@
       </c>
       <c r="I40" s="12" t="inlineStr">
         <is>
-          <t>유준이는 색종이 공예를 하기 위해 N x N 크기의 격자 종이를 가지고 있습니다. N은 3의 거듭제곱($3^k$, 1 &lt;= k &lt;= 7)입니다.</t>
+          <t>유준이는 N x N 크기의 색종이를 가지고 놀고 있습니다. 종이의 모든 칸이 -1, 0, 1 중 같은 숫자로 채워져 있지 않다면, 가로와 세로를 각각 3등분하여 총 9개의 동일한 크기의 작은 종이로 자르고 이 과정을...</t>
         </is>
       </c>
     </row>
@@ -39727,7 +39667,7 @@
       </c>
       <c r="I41" s="17" t="inlineStr">
         <is>
-          <t>지아는 자료구조 시간에 이진 트리의 전위 순회(Preorder)와 중위 순회(Inorder) 결과를 전달받았습니다. 트리를 구성하는 모든 노드는 1부터 N까지 서로 다른 고유한 자연수 번호를 가지고 있습니다.</t>
+          <t>자료구조를 연구하는 지아는 어떤 이진 트리를 전위 순회(Preorder)한 결과와 중위 순회(Inorder)한 결과를 전달받았습니다. 전위 순회의 첫 번째 원소가 항상 서브트리의 루트임을 이용하고, 중위 순회에서 루...</t>
         </is>
       </c>
     </row>
@@ -39817,7 +39757,7 @@
       </c>
       <c r="I43" s="17" t="inlineStr">
         <is>
-          <t>나은이는 정보 동아리에서 0부터 N까지 N+1개의 원소로 구성된 집합들을 관리하고 있습니다. 처음에는 모든 원소가 각각 하나의 집합을 이룹니다.</t>
+          <t>나은이는 1부터 N까지의 원소들로 구성된 서로소 집합 자료구조를 공부하고 있습니다. 두 원소가 속한 집합을 합치는 연산(0 a b)과, 두 원소가 같은 집합에 속해 있는지 확인하는 연산(1 a b)이 질의 형태로 주...</t>
         </is>
       </c>
     </row>
@@ -39952,7 +39892,7 @@
       </c>
       <c r="I46" s="12" t="inlineStr">
         <is>
-          <t>시아는 R x C 크기의 지도에서 바다(0)와 육지(1)를 관리하는 국토 개발 프로젝트를 진행하고 있습니다. 상하좌우로 인접한 육지(1)들은 하나의 섬을 형성합니다.</t>
+          <t>해양 탐험가 시아는 군도에 위치한 N개의 섬들 사이에 다리를 놓는 작업을 진행하고 있습니다. 다리가 하나씩 건설될 때마다 두 섬이 속한 군집이 합쳐집니다. 시아를 도와 각 연결 쿼리 후 현재 독립적인 연결 컴포넌트의...</t>
         </is>
       </c>
     </row>
@@ -39997,7 +39937,7 @@
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>아린이는 교내 여러 동아리들의 연합 규모를 조사하고 있습니다. 교내에는 1부터 N까지 번호가 붙은 N명의 학생이 있습니다.</t>
+          <t>학생회장 아린이는 교내 N명의 학생들이 구성하는 동아리 연합 네트워크를 분석하고 있습니다. 친구 관계인 두 학생은 같은 동아리로 묶이며, 친구의 친구 역시 동일한 동아리에 속합니다. 모든 관계가 주어졌을 때 가장 구...</t>
         </is>
       </c>
     </row>
@@ -40052,12 +39992,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>지아</t>
         </is>
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
@@ -40087,7 +40027,7 @@
       </c>
       <c r="I49" s="17" t="inlineStr">
         <is>
-          <t>1부터 N까지의 숫자로 이루어진 순열이 주어졌을 때, 사전순으로 바로 다음에 오는 순열을 찾는 알고리즘을 구현합니다. 만약 이미 사전순으로 마지막 순열(내림차순)이라면 -1을 출력합니다.</t>
+          <t>보안 시스템 연구원 지아는 비밀번호 순열 목록에서 사전순으로 바로 다음에 오는 순열을 생성하는 인증 알고리즘을 개발 중이다. 1부터 N까지의 숫자로 이루어진 순열이 주어졌을 때, 사전순으로 바로 다음에 오는 순열을 ...</t>
         </is>
       </c>
     </row>
@@ -40142,12 +40082,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>하윤</t>
         </is>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D51" s="15" t="inlineStr">
@@ -40177,7 +40117,7 @@
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>N명의 사람(1번부터 N번)이 원형 테이블에 둘러앉습니다. 회전하여 일치하는 배치는 동일한 것으로 간주합니다.</t>
+          <t>연회 기획자 하윤이는 귀빈들을 원형 테이블에 둘러앉힐 때 서로 사이가 좋은 사람들끼리 이웃하도록 순열 좌석을 배치하고 있다. N명의 사람(1번부터 N번)이 원형 테이블에 둘러앉습니다.</t>
         </is>
       </c>
     </row>
@@ -40987,7 +40927,7 @@
       </c>
       <c r="I69" s="17" t="inlineStr">
         <is>
-          <t>프로게이머 서윤이는 실시간 전략 시뮬레이션 게임(RTS)에서 최고의 연구 빌드오더를 설계하고 있습니다. 게임 내에는 1번부터 N번까지 총 N개의 기술(Tech)이 존재합니다.</t>
+          <t>게임 개발자 서윤이는 전략 시뮬레이션 게임에서 건물이나 유닛을 생산하기 위한 테크트리 선행 관계를 정의하고 있습니다. 특정 기술을 연구하려면 선행 기술들이 모두 완료되어야 합니다. 주어진 선행 관계를 바탕으로 모든 ...</t>
         </is>
       </c>
     </row>
@@ -41032,7 +40972,7 @@
       </c>
       <c r="I70" s="12" t="inlineStr">
         <is>
-          <t>DJ 선우는 음악 스트리밍 파티를 위해 1번부터 N번까지 N곡으로 구성된 플레이리스트를 제작 중입니다. 선우는 곡의 분위기(BPM, Mood) 전개가 자연스럽도록 M개의 곡 순서 규칙을 정했습니다.</t>
+          <t>음악 스트리밍 DJ 선우는 청취자의 몰입도를 높이기 위해 곡 간의 자연스러운 흐름 선행 조건을 반영한 플레이리스트를 제작하려 합니다. 특정 곡 u는 반드시 곡 v보다 먼저 재생되어야 한다는 조건들을 모두 만족하는 유...</t>
         </is>
       </c>
     </row>
@@ -41077,7 +41017,7 @@
       </c>
       <c r="I71" s="17" t="inlineStr">
         <is>
-          <t>유주는 생일 선물로 거대한 로봇 레고 블록 키트를 선물 받았습니다. 키트에는 1번부터 N번까지의 부품들이 있으며, 설명서에는 M개의 선행 조립 관계(부품 u를 먼저 조립해야 부품 v를 결합할 수 있음)가 적혀 있습니...</t>
+          <t>조립 블록 마니아 유주는 N개의 부품으로 구성된 거대 로봇을 조립하고 있습니다. 특정 부품들은 다른 기본 부품들이 먼저 조립되어 결합되어야만 다음 조립이 가능합니다. 유주가 부품들을 올바른 순서대로 조립할 수 있도록...</t>
         </is>
       </c>
     </row>
@@ -41122,7 +41062,7 @@
       </c>
       <c r="I72" s="12" t="inlineStr">
         <is>
-          <t>소프트웨어 PM인 은우는 대규모 프로젝트의 스프린트 태스크들을 관리하고 있습니다. 프로젝트에는 1번부터 N번까지 N개의 단위 작업(Task)이 있으며, 작업 간의 의존 관계(Dependency) M개가 주어집니다.</t>
+          <t>프로젝트 매니저 은우는 소프트웨어 릴리스를 위해 N개의 하위 태스크를 계획하고 있습니다. 태스크 간의 선행 의존성(Dependency)을 해결하여 작업자들에게 순차적으로 배분할 수 있는 작업 실행 일정을 수립하십시오...</t>
         </is>
       </c>
     </row>
@@ -41257,7 +41197,7 @@
       </c>
       <c r="I75" s="17" t="inlineStr">
         <is>
-          <t>시우는 동아리 방의 네트워크를 재구축하기 위해 길이가 제각각인 K개의 랜선을 가지고 있습니다. 시우는 이 K개의 랜선을 잘라서 모두 같은 길이의 랜선 N개를 만들어야 합니다.</t>
+          <t>시우는 길이가 제각각인 K개의 랜선을 가지고 있습니다. 이 랜선들을 잘라서 모두 같은 길이의 랜선 N개를 만들고자 합니다. 자른 후 남은 랜선 조각은 버려집니다. 만들 수 있는 최대 랜선 길이를 이진 탐색(Upper...</t>
         </is>
       </c>
     </row>
@@ -41302,7 +41242,7 @@
       </c>
       <c r="I76" s="12" t="inlineStr">
         <is>
-          <t>은우는 목공 실습 시간에 필요한 목재 M미터를 구하기 위해 숲으로 갔습니다. 숲에는 일렬로 심어진 N그루의 나무가 있으며, 각 나무의 높이가 주어집니다.</t>
+          <t>은우는 목재 공장에서 벌목 작업을 하고 있습니다. N개의 나무들이 한 줄로 서 있고, 절단기의 높이를 H로 지정하면 H보다 높은 나무들의 윗부분이 잘려 나갑니다. 은우가 필요한 최소 M미터의 나무를 가져가기 위해 설...</t>
         </is>
       </c>
     </row>
@@ -41347,7 +41287,7 @@
       </c>
       <c r="I77" s="17" t="inlineStr">
         <is>
-          <t>국가 예산 관리자인 하윤이는 여러 지방 부처의 예산 요청을 심사하여 국가 총예산 범위 내에서 배정하려고 합니다. 각 부처는 필요한 예산 요청액을 제출했습니다.</t>
+          <t>재정 담당관 하윤이는 N개 지자체의 예산 요청을 심사하여 국가 총예산 M원 내에서 배정하고자 합니다. 모든 요청의 총합이 M 이하이면 요청한 금액을 그대로 배정하고, 초과하면 특정 상한액(Cap)을 정하여 상한액 이...</t>
         </is>
       </c>
     </row>
@@ -41572,7 +41512,7 @@
       </c>
       <c r="I82" s="12" t="inlineStr">
         <is>
-          <t>초등학생 이준이는 장난감 사각 블록을 가지고 프랙탈 카펫 패턴을 조립하고 있습니다. $3^K \times 3^K$ 크기의 정사각형 판에서, 정중앙의 $3^{K-1} \times 3^{K-1}$ 영역은 블록을 비워두고...</t>
+          <t>초등학생 이준이는 장난감 사각 블록을 가지고 프랙탈 카펫 패턴을 조립하고 있습니다. 3^K x 3^K 크기의 정사각형 판에서, 정중앙의 3^{K-1} x 3^{K-1} 영역은 블록을 비워두고, 나머지 8개의 영역은 ...</t>
         </is>
       </c>
     </row>
@@ -41717,12 +41657,12 @@
       </c>
       <c r="B86" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>서윤</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
@@ -41752,7 +41692,7 @@
       </c>
       <c r="I86" s="12" t="inlineStr">
         <is>
-          <t>짝수 N명의 사람이 모여 축구 시합을 하려고 합니다. N명을 정확히 N/2명씩 스타트 팀과 링크 팀으로 나눕니다. 사람 i와 j가 같은 팀에 속했을 때 팀에 더해지는 시너지 능력치 S_ij가 2차원 배열로 주어집니다...</t>
+          <t>체육대회 운영위원 서윤이는 전체 인원을 두 팀으로 공평하게 나눌 때 팀 간의 능력치 차이가 최소가 되는 최적의 조합을 찾고 있다. 짝수 N명의 사람이 모여 축구 시합을 하려고 합니다. N명을 정확히 N/2명씩 스타트...</t>
         </is>
       </c>
     </row>
@@ -41762,12 +41702,12 @@
       </c>
       <c r="B87" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="C87" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D87" s="15" t="inlineStr">
@@ -41797,7 +41737,7 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>과일 명품관에서 N가지 과일(1번부터 N번) 중 서로 다른 R개를 골라 고급 선물 바구니를 구성하려고 합니다 (순서 무관). 그런데 과일 전문가들의 연구에 따르면, 함께 담았을 때 숙성 가스나 향의 충돌로 맛을 해치...</t>
+          <t>수제 디저트 카페를 운영하는 시아는 매장의 대표 디저트 메뉴 중 조화로운 조합을 선택하여 한정판 선물 세트를 구성하려 한다. 과일 명품관에서 N가지 과일(1번부터 N번) 중 서로 다른 R개를 골라 고급 선물 바구니를...</t>
         </is>
       </c>
     </row>
@@ -41807,12 +41747,12 @@
       </c>
       <c r="B88" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>아린</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
@@ -41842,7 +41782,7 @@
       </c>
       <c r="I88" s="12" t="inlineStr">
         <is>
-          <t>1부터 N까지의 자연수 중 서로 다른 6개의 수를 뽑아 로또 번호 조합을 만듭니다. 이때 '행운의 조건'으로 홀수의 개수가 정확히 3개(짝수도 3개)이고, 6개 수의 총합이 S 이상이어야 합니다.</t>
+          <t>통계학 연구원 아린이는 추첨 번호 후보군 중에서 수학적 확률 조건에 맞는 행운의 번호 조합들을 체계적으로 추출하고 있다. 1부터 N까지의 자연수 중 서로 다른 6개의 수를 뽑아 로또 번호 조합을 만듭니다.</t>
         </is>
       </c>
     </row>
@@ -41942,12 +41882,12 @@
       </c>
       <c r="B91" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>로운</t>
         </is>
       </c>
       <c r="C91" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D91" s="15" t="inlineStr">
@@ -41977,7 +41917,7 @@
       </c>
       <c r="I91" s="17" t="inlineStr">
         <is>
-          <t>탕후루 가게에서 N가지 과일(1번부터 N번)을 중복을 허용하여 꼬치에 아래에서부터 차례로 K개를 꽂아 만듭니다. 첫 입부터 마지막 입까지 씹히는 과일의 순서가 중요합니다.</t>
+          <t>축제 부스를 맡은 나은이는 여러 종류의 과일을 중복을 허용하여 꼬치에 꽂아 다채로운 맛의 탕후루 순서를 만들고 있다. 탕후루 가게에서 N가지 과일(1번부터 N번)을 중복을 허용하여 꼬치에 아래에서부터 차례로 K개를 ...</t>
         </is>
       </c>
     </row>
@@ -42032,12 +41972,12 @@
       </c>
       <c r="B93" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>유주</t>
         </is>
       </c>
       <c r="C93" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D93" s="15" t="inlineStr">
@@ -42067,7 +42007,7 @@
       </c>
       <c r="I93" s="17" t="inlineStr">
         <is>
-          <t>신호등에는 R(빨강), G(초록), B(파랑) 3가지 색이 있습니다. K초 동안 매 초마다 한 가지 색을 켜는데, 에너지 효율을 위해 동일한 색이 연속으로 점등될 수 없습니다.</t>
+          <t>교통 안전 모니터링을 담당하는 유주는 교차로 신호등의 불빛 점등 신호 패턴을 중복순열 조합으로 분석하고 있다. 신호등에는 R(빨강), G(초록), B(파랑) 3가지 색이 있습니다.</t>
         </is>
       </c>
     </row>
@@ -42122,12 +42062,12 @@
       </c>
       <c r="B95" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이준</t>
         </is>
       </c>
       <c r="C95" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D95" s="15" t="inlineStr">
@@ -42157,7 +42097,7 @@
       </c>
       <c r="I95" s="17" t="inlineStr">
         <is>
-          <t>1부터 M까지의 눈금이 있는 M면체 주사위를 K번 던집니다 (중복 허용, 던지는 순서 있음). K번 던져 나온 모든 눈금의 합이 정확히 S가 되는 서로 다른 주사위 던지기 결과의 총수를 구하시오.</t>
+          <t>보드게임 제작자 이준이는 N개의 주사위를 굴렸을 때 나올 수 있는 모든 눈금의 순서쌍 중 특정 합을 만족하는 경우의 수를 집계하고 있다. 1부터 M까지의 눈금이 있는 M면체 주사위를 K번 던집니다 (중복 허용, 던지...</t>
         </is>
       </c>
     </row>
@@ -42257,12 +42197,12 @@
       </c>
       <c r="B98" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>도하</t>
         </is>
       </c>
       <c r="C98" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>남아</t>
         </is>
       </c>
       <c r="D98" s="10" t="inlineStr">
@@ -42292,7 +42232,7 @@
       </c>
       <c r="I98" s="12" t="inlineStr">
         <is>
-          <t>방정식 x_1 + x_2 + ... + x_N = K 를 만족하는 정수해의 개수를 구합니다. 단, 각 변수 x_i는 최소 L 이상이어야 합니다 (x_i &gt;= L).</t>
+          <t>수학 퀴즈 동아리의 도하는 음이 아닌 정수해를 구하는 연립 방정식 문제를 중복조합 원리로 풀어내는 프로그램을 작성하고 있다. 방정식 x_1 + x_2 + ... + x_N = K 를 만족하는 정수해의 개수를 구합니다...</t>
         </is>
       </c>
     </row>
@@ -42302,12 +42242,12 @@
       </c>
       <c r="B99" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>이서</t>
         </is>
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>여아</t>
         </is>
       </c>
       <c r="D99" s="15" t="inlineStr">
@@ -42337,7 +42277,7 @@
       </c>
       <c r="I99" s="17" t="inlineStr">
         <is>
-          <t>1부터 N까지의 자연수 중 중복을 허용하여 K개를 골라 비내림차순(a_1 &lt;= a_2 &lt;= ... &lt;= a_K) 수열을 만듭니다. 이 수열들 중 모든 원소의 합이 짝수인 수열의 총 개수를 구하시오.</t>
+          <t>음악 작곡가 이서는 피아노 건반의 음높이가 점점 낮아지지 않는 아름다운 멜로디 수열을 중복조합 원리로 생성하고 있다. 1부터 N까지의 자연수 중 중복을 허용하여 K개를 골라 비내림차순(a_1 &lt;= a_2 &lt;= ......</t>
         </is>
       </c>
     </row>
@@ -43883,7 +43823,7 @@
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>최장_증가_부분수열_LIS</t>
+          <t>파일_합치기_최소_비용</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -43903,12 +43843,12 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>DP/D4_DP_최장_증가_부분수열_LIS</t>
+          <t>DP/D4_DP_파일_합치기_최소_비용</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>크기가 N인 수열 A가 주어질 때, 원소들이 엄격하게 증가하는 부분 수열(Strictly Increasing Subsequence) 중 '가장 길이가 긴 수열'의 길이를 구해야 합니다. 1. 단순 DP로 O(N^2)...</t>
+          <t>소설의 여러 장(Chapter)이 각각 독립된 파일로 나누어져 있습니다. 두 개의 연속된 파일을 합쳐 하나의 임시 파일로 만들고, 이 임시 파일들을 다시 합치는 과정을 반복하여 최종 하나의 완성본 파일로 묶으려 합니...</t>
         </is>
       </c>
     </row>
@@ -44043,7 +43983,7 @@
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>이미 N개의 정점으로 구성된 최소 신장 트리(MST)가 완성되어 있으며, 기존 트리의 가중치 합은 initialWeight입니다. 여기에 새로운 간선 (u, v, w) 하나가 추가 제안되었습니다.</t>
+          <t>기존에 완성된 최소 신장 트리(MST)에 새로운 간선 (u, v, w)가 추가되면 정확히 하나의 단순 사이클이 형성됩니다. 트리의 연결성을 유지하면서 가중치 합을 최소로 유지하기 위해, 형성된 사이클 상에서 가장 가...</t>
         </is>
       </c>
     </row>
@@ -44133,7 +44073,7 @@
       </c>
       <c r="I23" s="17" t="inlineStr">
         <is>
-          <t>최소 병목 스패닝 트리(Minimum Bottleneck Spanning Tree, MBST)는 그래프의 모든 정점을 연결하는 스패닝 트리 중, 포함된 간선들 중 '가장 가중치가 큰 간선의 가중치(Max Edge W...</t>
+          <t>스패닝 트리의 간선들 중 '가장 비용이 큰 단일 간선의 가중치(병목 비용)'를 최소화하는 트리(Min-Bottleneck Spanning Tree, MBST)를 구하는 문제입니다. 크루스칼 알고리즘으로 구한 MST의...</t>
         </is>
       </c>
     </row>
@@ -44223,7 +44163,7 @@
       </c>
       <c r="I25" s="17" t="inlineStr">
         <is>
-          <t>2차원 평면 위에 N개의 행성 기지가 위치해 있습니다. 각 기지의 좌표는 (x, y) 정수 좌표로 주어집니다. 모든 두 행성 기지 (i, j) 사이에는 우주 터널을 뚫을 수 있으며, 두 기지를 연결하는 터널의 건설 ...</t>
+          <t>2차원 평면 위에 N개의 통신 관측소 좌표 (x_i, y_i)가 주어집니다. 두 관측소 사이를 유선 케이블로 연결할 때의 비용은 두 점 사이의 유클리드 거리(또는 거리의 제곱에 비례)입니다. 모든 관측소를 하나의 통...</t>
         </is>
       </c>
     </row>
@@ -44673,7 +44613,7 @@
       </c>
       <c r="I35" s="17" t="inlineStr">
         <is>
-          <t>$R \times C$ 크기의 미로 격자판이 있습니다. 각 칸은 빈 칸(0)이거나, 부술 수 있는 특수 방화벽(1)입니다.</t>
+          <t>R x C 크기의 미로 격자판이 있습니다. 각 칸은 빈 칸(0)이거나, 부술 수 있는 특수 방화벽(1)입니다.</t>
         </is>
       </c>
     </row>
@@ -44763,7 +44703,7 @@
       </c>
       <c r="I37" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 정수 수열 A와 임계값 K가 주어집니다. 수열의 연속된 부분 구간 $[left, right]$에 대하여, 구간 내의 최댓값과 최솟값의 차이가 K 이하인 구간을 '안정 구간'이라고 부릅니다:</t>
+          <t>길이가 N인 정수 수열 A와 임계값 K가 주어집니다. 수열의 연속된 부분 구간 [left, right]에 대하여, 구간 내의 최댓값과 최솟값의 차이가 K 이하인 구간을 '안정 구간'이라고 부릅니다:</t>
         </is>
       </c>
     </row>
@@ -45123,7 +45063,7 @@
       </c>
       <c r="I45" s="17" t="inlineStr">
         <is>
-          <t>크기가 N인 정수 배열에서 K번째(1-based)로 작은 원소를 찾는 문제입니다. 전체 배열을 정렬하면 $O(N \log N)$이 걸리지만, 퀵소트(Quick Sort)의 분할 정복 기법을 변형한 퀵 셀렉트(Quic...</t>
+          <t>정렬되지 않은 N개의 데이터에서 K번째로 작은 원소를 정렬 없이 평균 O(N) 시간에 찾아내는 퀵셀렉트(Quickselect) 알고리즘입니다. 피벗(Pivot)을 기준으로 파티셔닝을 수행한 후, K의 위치가 속한 분...</t>
         </is>
       </c>
     </row>
@@ -45168,7 +45108,7 @@
       </c>
       <c r="I46" s="12" t="inlineStr">
         <is>
-          <t>길이가 N인 수열 A에서 $i &lt; j$이면서 $A[i] &gt; A[j]$인 쌍 $(i, j)$를 '역순쌍(Inversion)'이라고 합니다. 단순 이중 반복문으로 역순쌍을 셀 경우 $O(N^2)$ 시간이 걸려 $N=10...</t>
+          <t>크기 N인 배열 A에서 i &lt; j 이지만 A[i] &gt; A[j]를 만족하는 쌍 (i, j)를 역순쌍(Inversion)이라고 합니다. 단순 이중 루프 O(N^2)로는 100,000 크기의 배열을 처리할 수 없으므로, ...</t>
         </is>
       </c>
     </row>
@@ -45213,7 +45153,7 @@
       </c>
       <c r="I47" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 정수 배열 A에서 연속된 부분 배열(Subarray)의 합 중 최댓값을 구하는 문제입니다. (적어도 하나의 원소는 선택해야 합니다.) 이 문제는 대표적인 분할 정복(Divide and Conquer) 응...</t>
+          <t>연속된 부분 배열의 원소 합 중 최댓값을 구하는 문제입니다. 배열을 좌우 두 영역으로 나누어, 1) 왼쪽 영역의 최대 부분합, 2) 오른쪽 영역의 최대 부분합, 3) 중앙 경계를 가로지르는 최대 부분합을 각각 분할 ...</t>
         </is>
       </c>
     </row>
@@ -45258,7 +45198,7 @@
       </c>
       <c r="I48" s="12" t="inlineStr">
         <is>
-          <t>피보나치 수열은 $F_0 = 0, F_1 = 1$, 그리고 $N \ge 2$에 대해 $F_N = F_{N-1} + F_{N-2}$로 정의됩니다. $N$이 매우 클 때(최대 $10^{16}$), 동적 계획법(DP)으로...</t>
+          <t>피보나치 수열의 N번째 항 F_N을 구하는 문제입니다. N이 10^18까지 주어지므로 동적 계획법 O(N)으로도 해결할 수 없습니다. 상태 전이 행렬 [[1, 1], [1, 0]]의 N제곱을 분할 정복(Matrix ...</t>
         </is>
       </c>
     </row>
@@ -45393,7 +45333,7 @@
       </c>
       <c r="I51" s="17" t="inlineStr">
         <is>
-          <t>가중치 유니온 파인드(Weighted Union-Find)는 각 원소 간의 상대적 차이(Potential Difference)를 추적할 수 있는 확장 자료구조입니다. 연구소에서 N개의 물건의 무게를 비교하고 있습니다...</t>
+          <t>각 정점 x, y 사이의 상대적 무게 차이(weight[y] - weight[x] = w)를 유지하고 질의하는 문제입니다. 경로 압축 시 루트와의 상대 오프셋(Potential)을 누적 갱신하여, 두 원소 간의 무게...</t>
         </is>
       </c>
     </row>
@@ -45483,7 +45423,7 @@
       </c>
       <c r="I53" s="17" t="inlineStr">
         <is>
-          <t>서로소 집합은 집합을 합치는(Union) 연산은 매우 빠르지만, 이미 합쳐진 집합을 쪼개거나 간선을 제거하는 연산은 직접 지원하지 않습니다. 따라서 간선이 시간 순서대로 제거되는 문제는 질의를 끝에서부터 거꾸로 역순...</t>
+          <t>그래프에서 간선이 하나씩 '제거'되는 상황에서의 연결성 질의는 일반적인 유니온파인드로 직접 처리하기 어렵습니다. 쿼리를 모두 수집한 뒤, 모든 간선이 제거된 최종 상태에서 역순(시간 역류)으로 간선을 '추가(Unio...</t>
         </is>
       </c>
     </row>
@@ -45528,7 +45468,7 @@
       </c>
       <c r="I54" s="12" t="inlineStr">
         <is>
-          <t>두 팀으로 나누어 시합을 하려고 합니다. 일부 참가자 쌍 사이에 '적대 관계'가 주어집니다.</t>
+          <t>정점 u와 v가 서로 다른 색으로 칠해져야 한다는 조건들이 동적으로 추가될 때, 그래프가 이분 그래프(Bipartite Graph)로 유지되는지 실시간으로 판별합니다. 각 원소 x에 대해 동치 관계 x와 반대 관계 ...</t>
         </is>
       </c>
     </row>
@@ -45573,7 +45513,7 @@
       </c>
       <c r="I55" s="17" t="inlineStr">
         <is>
-          <t>초기에 1부터 N까지 N개의 단독 노드로 이루어진 시스템이 있습니다. 네트워크 간선이 하나씩 순차적으로 추가될 때마다, 전체 네트워크에서 '가장 큰 연결 컴포넌트(Maximum Connected Component)의...</t>
+          <t>N개의 정점이 있는 무방향 그래프에서 간선이 하나씩 추가될 때마다, 전체 그래프에서 가장 원소 수가 많은 연결 컴포넌트의 크기(최댓값)를 즉각 반환하는 동적 질의 문제입니다. 각 집합의 크기를 루트 노드에 저장하고 ...</t>
         </is>
       </c>
     </row>
@@ -45728,7 +45668,7 @@
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>과일트럭_최단배달</t>
+          <t>N자리_순열_사전순_K번째_복원</t>
         </is>
       </c>
       <c r="E59" s="13" t="inlineStr">
@@ -45748,12 +45688,12 @@
       </c>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>순열/D4_순열_과일트럭_최단배달</t>
+          <t>순열/D4_순열_N자리_순열_사전순_K번째_복원</t>
         </is>
       </c>
       <c r="I59" s="17" t="inlineStr">
         <is>
-          <t>신선 과일 배송 트럭이 과일 유통센터(0번)에서 출발하여 N개의 가맹 과일 매장(1번부터 N번)을 모두 정확히 한 번씩 방문하여 배송을 마친 뒤, 다시 유통센터(0번)로 복귀해야 합니다. 지점 i에서 지점 j로 이동...</t>
+          <t>1부터 N까지의 자연수를 한 번씩만 사용하여 만들 수 있는 N!개의 순열들을 사전순으로 정렬했을 때, K번째로 오는 순열을 복원하는 문제입니다. N이 최대 20에 달할 수 있으므로 N! = 2.4 x 10^18로 모...</t>
         </is>
       </c>
     </row>
@@ -45773,7 +45713,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>부등호_관계식_최대_최소_수열</t>
+          <t>과일트럭_최단배달</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
@@ -45793,12 +45733,12 @@
       </c>
       <c r="H60" s="12" t="inlineStr">
         <is>
-          <t>순열/D4_순열_부등호_관계식_최대_최소_수열</t>
+          <t>순열/D4_순열_과일트럭_최단배달</t>
         </is>
       </c>
       <c r="I60" s="12" t="inlineStr">
         <is>
-          <t>주어진 부등호 관계식을 만족하는 k+1자리의 최대 정수와 최소 정수를 각각 문자열 형태로 한 줄씩 출력하십시오.</t>
+          <t>신선 과일 배송 트럭이 과일 유통센터(0번)에서 출발하여 N개의 가맹 과일 매장(1번부터 N번)을 모두 정확히 한 번씩 방문하여 배송을 마친 뒤, 다시 유통센터(0번)로 복귀해야 합니다. 지점 i에서 지점 j로 이동...</t>
         </is>
       </c>
     </row>
@@ -45818,7 +45758,7 @@
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>부등호_수열_생성</t>
+          <t>부등호_관계식_최대_최소_수열</t>
         </is>
       </c>
       <c r="E61" s="13" t="inlineStr">
@@ -45838,12 +45778,12 @@
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>순열/D4_순열_부등호_수열_생성</t>
+          <t>순열/D4_순열_부등호_관계식_최대_최소_수열</t>
         </is>
       </c>
       <c r="I61" s="17" t="inlineStr">
         <is>
-          <t>k개의 부등호 기호('&lt;', '&gt;')가 나열된 순열이 주어집니다. 0부터 9까지의 서로 다른 숫자 k+1개를 골라 부등호 관계를 모두 만족하도록 배치하여 k+1자리 정수를 만듭니다.</t>
+          <t>주어진 부등호 관계식을 만족하는 k+1자리의 최대 정수와 최소 정수를 각각 문자열 형태로 한 줄씩 출력하십시오.</t>
         </is>
       </c>
     </row>
@@ -46203,7 +46143,7 @@
       </c>
       <c r="I69" s="17" t="inlineStr">
         <is>
-          <t>길이가 N인 수열 A와 윈도우 크기 L이 주어집니다. 수열에서 $i = 0$부터 $N - L$까지 각 윈도우 $[i, i + L - 1]$의 최솟값을 모두 구해야 합니다.</t>
+          <t>길이가 N인 수열 A와 윈도우 크기 L이 주어집니다. 수열에서 i = 0부터 N - L까지 각 윈도우 [i, i + L - 1]의 최솟값을 모두 구해야 합니다.</t>
         </is>
       </c>
     </row>
@@ -46563,7 +46503,7 @@
       </c>
       <c r="I77" s="17" t="inlineStr">
         <is>
-          <t>1번부터 N번까지의 사람이 원형으로 둘러앉아 있을 때, 순서대로 K번째 사람을 탈락시키는 요세푸스 순열 문제입니다. 일반적인 배열이나 단순 큐를 사용할 경우 $K$가 매우 크거나 노드 삭제가 빈번할 때 $O(N \t...</t>
+          <t>1번부터 N번까지의 사람이 원형으로 둘러앉아 있을 때, 순서대로 K번째 사람을 탈락시키는 요세푸스 순열 문제입니다. 일반적인 배열이나 단순 큐를 사용할 경우 K가 매우 크거나 노드 삭제가 빈번할 때 O(N x K)의...</t>
         </is>
       </c>
     </row>
@@ -46653,7 +46593,7 @@
       </c>
       <c r="I79" s="17" t="inlineStr">
         <is>
-          <t>전략 시뮬레이션 게임에서 건물 1번부터 N번까지 각각을 짓는 데 걸리는 건설 시간 time[i]가 주어집니다. 또한 건물 간의 선행 건설 조건 M개가 주어집니다.</t>
+          <t>건물을 짓는 데 걸리는 시간 D_i와 건물 간의 선행 건설 규칙이 주어집니다. 여러 건물을 동시에 병렬로 지을 수 있을 때, 특정 목표 건물 W를 완성하기까지 걸리는 최소 총 소요 시간을 구하는 문제입니다. 진입 차...</t>
         </is>
       </c>
     </row>
@@ -46698,7 +46638,7 @@
       </c>
       <c r="I80" s="12" t="inlineStr">
         <is>
-          <t>방향 그래프가 주어졌을 때, 위상 정렬의 가능한 결과가 다음 세 가지 중 어느 것에 해당하는지 판별하는 문제입니다: 1. "CYCLE": 그래프에 사이클이 존재하여 위상 정렬이 불가능한 경우</t>
+          <t>주어진 방향 그래프의 위상 정렬 순서가 '유일하게 단 하나만 존재하는지(Unique)', '여러 가지 순서가 가능한지(Multiple)', 아니면 '사이클이 발생하여 불가능한지(Cycle)'를 판별하는 고난도 알고리...</t>
         </is>
       </c>
     </row>
@@ -46743,7 +46683,7 @@
       </c>
       <c r="I81" s="17" t="inlineStr">
         <is>
-          <t>민우는 1번부터 N번까지 총 N개의 문제로 구성된 문제집을 풀려고 합니다. 문제들은 난이도 순서대로 1번이 가장 쉽고 N번이 가장 어렵습니다.</t>
+          <t>N개의 문제를 풀어야 합니다. 문제 간에 먼저 풀어야 하는 선행 조건이 주어지고, 선행 조건이 없는 문제들 중에서는 번호가 작은 문제를 먼저 푸는 것이 좋습니다. 일반 큐 대신 최소 힙(Min-PriorityQueu...</t>
         </is>
       </c>
     </row>
@@ -46763,7 +46703,7 @@
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>임계_경로_최장_소요_시간</t>
+          <t>사전순_가장_앞선_위상정렬</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
@@ -46783,12 +46723,12 @@
       </c>
       <c r="H82" s="12" t="inlineStr">
         <is>
-          <t>위상정렬/D4_위상정렬_임계_경로_최장_소요_시간</t>
+          <t>위상정렬/D4_위상정렬_사전순_가장_앞선_위상정렬</t>
         </is>
       </c>
       <c r="I82" s="12" t="inlineStr">
         <is>
-          <t>임계 경로(Critical Path) 기법은 대규모 건설 및 소프트웨어 프로젝트에서 전체 작업이 완료되는 최단 완료 시간(즉, 선행 제약으로 인한 최장 경로의 길이)을 계산하는 핵심 알고리즘입니다. 프로젝트의 각 작...</t>
+          <t>N개의 문제로 구성된 알고리즘 문제집이 있습니다. 각 문제는 1번부터 N번까지 번호가 매겨져 있습니다. 문제들 사이에는 특정 문제를 다른 문제보다 먼저 푸는 것이 좋은 M개의 선행 규칙이 주어집니다.</t>
         </is>
       </c>
     </row>
@@ -46808,7 +46748,7 @@
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>임계경로_작업_스케줄러</t>
+          <t>임계_경로_최장_소요_시간</t>
         </is>
       </c>
       <c r="E83" s="13" t="inlineStr">
@@ -46828,12 +46768,12 @@
       </c>
       <c r="H83" s="17" t="inlineStr">
         <is>
-          <t>위상정렬/D4_위상정렬_임계경로_작업_스케줄러</t>
+          <t>위상정렬/D4_위상정렬_임계_경로_최장_소요_시간</t>
         </is>
       </c>
       <c r="I83" s="17" t="inlineStr">
         <is>
-          <t>대형 건설 프로젝트에는 1번부터 N번까지 총 N개의 작업이 있습니다. 각 작업 i는 완료하는 데 t_i 시간이 소요되며, 작업들 간의 선후 관계가 방향 비순환 그래프(DAG)로 주어집니다.</t>
+          <t>대규모 건설 프로젝트에서 전체 공정이 완료되는 최소 시간(즉, 시작점에서 도착점까지의 최장 경로)을 계산하고, 이 완료 시간에 직접적인 영향을 미치는 임계 경로 간선들의 총 개수를 역추적(Backtracking)하여...</t>
         </is>
       </c>
     </row>
@@ -46878,7 +46818,7 @@
       </c>
       <c r="I84" s="12" t="inlineStr">
         <is>
-          <t>크기가 N x N인 2차원 배열 A가 있습니다. 배열의 각 행과 열은 1부터 시작하며, A[i][j] = i * j 입니다. 이 수를 1차원 배열 B에 모두 넣으면 크기가 N^2인 배열이 됩니다.</t>
+          <t>N x N 크기의 2차원 배열 A의 각 원소는 A[i][j] = i * j 입니다. 이 수들을 1차원 배열 B에 넣고 오름차순 정렬했을 때, B[K]번째에 위치하는 수를 구하는 문제입니다. N이 최대 10^5로 N^...</t>
         </is>
       </c>
     </row>
@@ -47013,7 +46953,7 @@
       </c>
       <c r="I87" s="17" t="inlineStr">
         <is>
-          <t>보석 상자에 M가지 서로 다른 색상의 보석이 들어 있습니다. i번째 색상의 보석은 count[i]개 존재합니다.</t>
+          <t>M가지 색상의 보석들이 각각 몇 개씩 주어지고, N명의 학생들에게 보석을 나누어 주려고 합니다. 각 학생은 한 가지 색상의 보석만 받을 수 있으며, 받지 못하는 학생이 있어도 됩니다. 가장 많은 보석을 받은 학생이 ...</t>
         </is>
       </c>
     </row>
@@ -47058,7 +46998,7 @@
       </c>
       <c r="I88" s="12" t="inlineStr">
         <is>
-          <t>국제공항 입국심사대에서 N명의 심사관이 대기 중인 M명의 승객을 심사하려고 합니다. 각 심사관마다 한 명의 승객을 심사하는 데 걸리는 시간(times[i])이 제각기 다릅니다.</t>
+          <t>입국 심사대 N개가 있고 각 심사관마다 한 사람을 심사하는 데 걸리는 시간 T_k가 다릅니다. 심사를 기다리는 입국자 M명이 있을 때, 모든 사람이 심사를 완료하는 데 걸리는 최소 총 소요 시간을 구하십시오. 시간 ...</t>
         </is>
       </c>
     </row>
@@ -47148,7 +47088,7 @@
       </c>
       <c r="I90" s="12" t="inlineStr">
         <is>
-          <t>한 변의 길이가 $2^N$인 2차원 배열을 'Z' 모양으로 재귀 탐색합니다. $2 \times 2$ 배열에서는 왼쪽 위(0) -&gt; 오른쪽 위(1) -&gt; 왼쪽 아래(2) -&gt; 오른쪽 아래(3) 순서로 방문합니다.</t>
+          <t>한 변의 길이가 2^N인 2차원 배열을 'Z' 모양으로 재귀 탐색합니다. 2 x 2 배열에서는 왼쪽 위(0) -&gt; 오른쪽 위(1) -&gt; 왼쪽 아래(2) -&gt; 오른쪽 아래(3) 순서로 방문합니다.</t>
         </is>
       </c>
     </row>
@@ -47193,7 +47133,7 @@
       </c>
       <c r="I91" s="17" t="inlineStr">
         <is>
-          <t>크기 $3^K \times 3^K$의 시에르핀스키 카펫 격자를 재귀적으로 생성하는 문제입니다. $K=1$인 경우 가운데 한 칸이 공백이고 주변 8칸이 별('*')인 패턴입니다:</t>
+          <t>크기 3^K x 3^K의 시에르핀스키 카펫 격자를 재귀적으로 생성하는 문제입니다. K=1인 경우 가운데 한 칸이 공백이고 주변 8칸이 별('*')인 패턴입니다:</t>
         </is>
       </c>
     </row>
@@ -47238,7 +47178,7 @@
       </c>
       <c r="I92" s="12" t="inlineStr">
         <is>
-          <t>$N \times N$ ($N = 2^K$) 크기의 흑백 영상이 주어집니다. 각 픽셀은 흰색(0) 또는 검은색(1)입니다. 쿼드 트리(Quad Tree) 알고리즘을 사용하여 영상을 다음과 같이 재귀적으로 압축합니다:</t>
+          <t>N x N (N = 2^K) 크기의 흑백 영상이 주어집니다. 각 픽셀은 흰색(0) 또는 검은색(1)입니다. 쿼드 트리(Quad Tree) 알고리즘을 사용하여 영상을 다음과 같이 재귀적으로 압축합니다:</t>
         </is>
       </c>
     </row>
@@ -47328,7 +47268,7 @@
       </c>
       <c r="I94" s="12" t="inlineStr">
         <is>
-          <t>세 개의 기둥(1번, 2번, 3번)과 크기가 서로 다른 N개의 원판이 1번 기둥에 꽂혀 있습니다. 하노이의 탑 규칙에 따라 모든 원판을 3번 기둥으로 옮기려면 총 $2^N - 1$번의 이동이 필요합니다.</t>
+          <t>세 개의 기둥(1번, 2번, 3번)과 크기가 서로 다른 N개의 원판이 1번 기둥에 꽂혀 있습니다. 하노이의 탑 규칙에 따라 모든 원판을 3번 기둥으로 옮기려면 총 2^N - 1번의 이동이 필요합니다.</t>
         </is>
       </c>
     </row>
@@ -47438,7 +47378,7 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t>스타트와_링크_팀_밸런스_최적화</t>
+          <t>도심_스프링클러_최적_감시_배치</t>
         </is>
       </c>
       <c r="E97" s="13" t="inlineStr">
@@ -47458,12 +47398,12 @@
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>조합/D4_조합_스타트와_링크_팀_밸런스_최적화</t>
+          <t>조합/D4_조합_도심_스프링클러_최적_감시_배치</t>
         </is>
       </c>
       <c r="I97" s="17" t="inlineStr">
         <is>
-          <t>주어진 능력치 행렬 S에 대해 스타트 팀과 링크 팀의 능력치 차이의 최솟값을 구하십시오.</t>
+          <t>도시 방재 본부에서는 N x N 크기의 도심 구역에서 화재 위험이 있는 잔디/건물 구역 H곳을 보호하기 위해, K개의 후보 위치 중 정확히 M개의 자동 스프링클러를 설치하려고 합니다. 각 보호 구역 h와 스프링클러 ...</t>
         </is>
       </c>
     </row>
@@ -47483,7 +47423,7 @@
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>치킨_배달_거리_최적화</t>
+          <t>스타트와_링크_팀_밸런스_최적화</t>
         </is>
       </c>
       <c r="E98" s="13" t="inlineStr">
@@ -47503,12 +47443,12 @@
       </c>
       <c r="H98" s="12" t="inlineStr">
         <is>
-          <t>조합/D4_조합_치킨_배달_거리_최적화</t>
+          <t>조합/D4_조합_스타트와_링크_팀_밸런스_최적화</t>
         </is>
       </c>
       <c r="I98" s="12" t="inlineStr">
         <is>
-          <t>주어진 도시 지도에서 치킨집 최대 M개를 남겼을 때 얻을 수 있는 도시의 최소 치킨 거리를 구하십시오.</t>
+          <t>주어진 능력치 행렬 S에 대해 스타트 팀과 링크 팀의 능력치 차이의 최솟값을 구하십시오.</t>
         </is>
       </c>
     </row>
@@ -47528,7 +47468,7 @@
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>치킨거리_최소화</t>
+          <t>치킨_배달_거리_최적화</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
@@ -47548,12 +47488,12 @@
       </c>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>조합/D4_조합_치킨거리_최소화</t>
+          <t>조합/D4_조합_치킨_배달_거리_최적화</t>
         </is>
       </c>
       <c r="I99" s="17" t="inlineStr">
         <is>
-          <t>N x N 크기의 도시에 집(1)과 치킨집(2)이 있습니다. 도시의 치킨집 중 최대 M개만을 남기고 나머지는 폐업시키려 합니다.</t>
+          <t>주어진 도시 지도에서 치킨집 최대 M개를 남겼을 때 얻을 수 있는 도시의 최소 치킨 거리를 구하십시오.</t>
         </is>
       </c>
     </row>
@@ -48068,7 +48008,7 @@
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>벨만포드_음수_사이클_검출</t>
+          <t>다익스트라_최단경로_역추적_복원</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr">
@@ -48088,12 +48028,12 @@
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>최단경로/D4_최단경로_벨만포드_음수_사이클_검출</t>
+          <t>최단경로/D4_최단경로_다익스트라_최단경로_역추적_복원</t>
         </is>
       </c>
       <c r="I111" s="17" t="inlineStr">
         <is>
-          <t>1번 도시에서 출발하여 도달 가능한 음수 사이클이 있으면 -1을 출력하고, 없으면 2번부터 N번 도시까지의 최단 거리를 한 줄에 하나씩 출력하십시오.</t>
+          <t>N개의 도시와 도시 사이를 잇는 M개의 일방통행 유료 버스 노선이 있습니다. 출발 도시 S에서 도착 도시 E까지 이동하는 최소 비용을 계산하고, 그 최소 비용을 달성하는 실제 최단 경로 상의 방문 도시 순서를 역추적...</t>
         </is>
       </c>
     </row>
@@ -48113,7 +48053,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>벨만포드_타임머신_탐색</t>
+          <t>벨만포드_음수_사이클_검출</t>
         </is>
       </c>
       <c r="E112" s="13" t="inlineStr">
@@ -48133,12 +48073,12 @@
       </c>
       <c r="H112" s="12" t="inlineStr">
         <is>
-          <t>최단경로/D4_최단경로_벨만포드_타임머신_탐색</t>
+          <t>최단경로/D4_최단경로_벨만포드_음수_사이클_검출</t>
         </is>
       </c>
       <c r="I112" s="12" t="inlineStr">
         <is>
-          <t>N개의 도시가 있고, 도시 사이를 이동하는 M개의 버스 노선이 있습니다. 각 버스 노선은 출발 도시 u, 도착 도시 v, 그리고 이동 시간 w를 갖습니다.</t>
+          <t>1번 도시에서 출발하여 도달 가능한 음수 사이클이 있으면 -1을 출력하고, 없으면 2번부터 N번 도시까지의 최단 거리를 한 줄에 하나씩 출력하십시오.</t>
         </is>
       </c>
     </row>
@@ -48428,7 +48368,7 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>이중_우선순위_큐_커스텀_구현</t>
+          <t>우선순위큐_중앙값_실시간_추적</t>
         </is>
       </c>
       <c r="E119" s="13" t="inlineStr">
@@ -48448,12 +48388,12 @@
       </c>
       <c r="H119" s="17" t="inlineStr">
         <is>
-          <t>큐/D4_큐_이중_우선순위_큐_커스텀_구현</t>
+          <t>큐/D4_큐_우선순위큐_중앙값_실시간_추적</t>
         </is>
       </c>
       <c r="I119" s="17" t="inlineStr">
         <is>
-          <t>주어진 N개의 연산을 모두 수행한 후, 큐가 비어있으면 "EMPTY"를 출력하고, 비어있지 않다면 최댓값과 최솟값을 공백으로 구분하여 출력하십시오.</t>
+          <t>빅데이터 스트리밍 관제 시스템에서 정수 데이터가 실시간으로 하나씩 순차 입력됩니다. 수가 하나씩 추가될 때마다 지금까지 입력된 수들 중 '중앙값(Median)'을 즉시 계산해야 합니다.</t>
         </is>
       </c>
     </row>
@@ -48473,7 +48413,7 @@
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>트럭의_다리_건너기</t>
+          <t>이중_우선순위_큐_커스텀_구현</t>
         </is>
       </c>
       <c r="E120" s="13" t="inlineStr">
@@ -48493,12 +48433,12 @@
       </c>
       <c r="H120" s="12" t="inlineStr">
         <is>
-          <t>큐/D4_큐_트럭의_다리_건너기</t>
+          <t>큐/D4_큐_이중_우선순위_큐_커스텀_구현</t>
         </is>
       </c>
       <c r="I120" s="12" t="inlineStr">
         <is>
-          <t>길이가 W이고 최대 하중 L까지 견딜 수 있는 일차선 다리가 있습니다. N대의 트럭이 정해진 순서대로 다리를 건너려고 합니다. 각 트럭의 무게는 A_1, A_2, ..., A_N입니다.</t>
+          <t>주어진 N개의 연산을 모두 수행한 후, 큐가 비어있으면 "EMPTY"를 출력하고, 비어있지 않다면 최댓값과 최솟값을 공백으로 구분하여 출력하십시오.</t>
         </is>
       </c>
     </row>

</xml_diff>